<commit_message>
sync(excel): update Master_Health_Articles_MVP and roadmaps with latest web content and canonical clinical sources
</commit_message>
<xml_diff>
--- a/docs/Master_Health_Articles_MVP - 30 Blog Topics.xlsx
+++ b/docs/Master_Health_Articles_MVP - 30 Blog Topics.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28000" windowHeight="16360" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Master_Health_Articles_MVP - 30" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master_Health_Articles_MVP - 30" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1295,7 +1295,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L34"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.4375" defaultRowHeight="16.8"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.4375" defaultRowHeight="16.8" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" style="1" min="1" max="1"/>
     <col width="24" customWidth="1" style="1" min="2" max="2"/>
@@ -1418,12 +1418,12 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Decoding Your Menstrual Cycle: Beyond Just Your Period</t>
+          <t>The 4 Phases of Your Menstrual Cycle: How Hormones Shape Your Energy, Sleep, and Wearable Biometrics</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Giải Mã Chu Kỳ Kinh Nguyệt: Chiếc Đồng Hồ Sinh Học Thứ Hai Của Phái Đẹp</t>
+          <t>4 Giai Đoạn Của Chu Kỳ Kinh Nguyệt: Cách Hormone Điều Phối Năng Lượng, Giấc Ngủ Và Chỉ Số Sinh Học Trên Thiết Bị Đeo</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>The 4 Phases of Your Cycle: How Hormones Direct Energy, Metabolism &amp; Mood</t>
+          <t>The 4 Phases of Your Menstrual Cycle: How Hormones Shape Your Energy, Sleep, and Wearable Biometrics</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>4 Giai Đoạn Chu Kỳ Kinh Nguyệt: Cách Hormone Điều Phối Năng Lượng, Giấc Ngủ &amp; Chỉ Số Sinh Học</t>
+          <t>4 Giai Đoạn Của Chu Kỳ Kinh Nguyệt: Cách Hormone Điều Phối Năng Lượng, Giấc Ngủ Và Chỉ Số Sinh Học Trên Thiết Bị Đeo</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Demystifying Menstrual Cramps &amp; Fatigue: Science-Backed Relief Protocols</t>
+          <t>PMS, Cramps, and Luteal Cravings: The Neuro-Endocrine Science &amp; Targeted Nutrition Protocol</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Hóa Giải Đau Bụng Kinh, Mệt Mỏi &amp; Đầy Hơi: Khoa Học Giảm Đau Chuẩn Y Khoa</t>
+          <t>Hội Chứng Tiền Kinh Nguyệt (PMS), Đau Bụng Kinh &amp; Cơn Thèm Ăn Pha Hoàng Thể: Khoa Học Thần Kinh – Nội Tiết Và Phác Đồ Dinh Dưỡng</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -1608,12 +1608,12 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Nghiên cứu từ hơn 600.000 chu kỳ cho thấy chỉ 13% phụ nữ có chu kỳ đúng 28 ngày. Khám phá cách thuật toán thiết bị đeo nhận diện chu kỳ anovulatory và ranh giới giữa dao động tự nhiên với bệnh lý.</t>
+          <t>Nghiên cứu quy mô lớn từ hơn 600.000 chu kỳ đăng trên tạp chí npj Digital Medicine cho thấy chỉ có khoảng 13% phụ nữ có chu kỳ đúng 28 ngày chuẩn mực. Khám phá cách các thuật toán thiết bị đeo (như Apple Health và WHOOP) nhận diện chu kỳ không rụng trứng (Anovulatory), phân biệt sự dao động sinh lý tự nhiên với các dấu hiệu cảnh báo bệnh lý cần thăm khám y khoa.</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>Dao động chu kỳ trong biên độ ±2 đến 4 ngày là hoàn toàn bình thường. Cần đi khám nếu chu kỳ ngắn hơn 21 ngày, dài hơn 35 ngày hoặc độ dài trồi sụt trên 8 ngày giữa các tháng.</t>
+          <t>Dao động chu kỳ trong biên độ ±2 đến 4 ngày giữa các tháng là hoàn toàn khỏe mạnh. Bạn chỉ cần thăm khám y tế khi chu kỳ ngắn hơn 21 ngày, dài hơn 35 ngày liên tục, độ dài trồi sụt trên 8–10 ngày, hoặc thiếu bước nhảy thân nhiệt cơ bản (+0.3°C) ở nửa sau chu kỳ.</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
@@ -1658,12 +1658,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>The 6-Day Fertile Window: Biological Timing, LH Surge &amp; Wearable Clues</t>
+          <t>The 6-Day Fertile Window: The Exact Biological Timeline of Conception &amp; Multi-Sensor Tracking</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Cửa Sổ Thụ Thai 6 Ngày: Dòng Thời Gian Sinh Học Chuẩn Xác Của Sự Thụ Tinh &amp; Đỉnh Rụng Trứng</t>
+          <t>Cửa Sổ Thụ Thai 6 Ngày: Dòng Thời Gian Sinh Học Chính Xác Của Sự Thụ Tinh &amp; Theo Dõi Đa Cảm Biến</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -1728,12 +1728,12 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Estrogen và Progesterone không chỉ chi phối tử cung mà còn gắn với các thụ thể ERα, ERβ và PR khắp cơ thể, điều tiết huyết áp, mật độ xương, chuyển hóa đường huyết và khả năng phục hồi thần kinh.</t>
+          <t>Estrogen và Progesterone không chỉ điều khiển niêm mạc tử cung mà còn gắn kết với hàng triệu thụ thể chuyên biệt tại mạch máu, khung xương, tế bào thần kinh và cơ bắp. Khám phá cách hai hormone quyền lực này định hình huyết áp, khả năng phục hồi thần kinh tự chủ (HRV) và tốc độ trao đổi chất của bạn qua từng tuần.</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>Estrogen là hormone bảo vệ tim mạch, tăng giãn mạch và thúc đẩy đồng hóa cơ bắp; trong khi Progesterone nâng nhiệt độ cơ sở, tăng dị hóa protein và tăng phân giải axit béo ở nửa cuối chu kỳ.</t>
+          <t>Estrogen là hormone bảo vệ tim mạch, tăng độ đàn hồi mạch máu và thúc đẩy đồng hóa cơ bắp; trong khi Progesterone nâng nhiệt độ cơ sở lõi, tăng phân giải axit béo và kích thích hô hấp ở nửa sau chu kỳ. Đừng cố gắng duy trì cùng một giáo án dinh dưỡng và luyện tập khi tỷ lệ E2:P4 thay đổi.</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
@@ -1788,12 +1788,12 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Estrogen kích hoạt tổng hợp serotonin và dopamine tại vỏ não trước trán mang lại cảm giác hưng phấn; khi cả hai hormone sụt giảm trước kỳ kinh, nồng độ allopregnanolone tụt dốc gây bất an và giảm động lực.</t>
+          <t>Sự thăng trầm của cảm xúc trong tháng không bắt nguồn từ sự yếu đuối tâm lý—đó là hệ quả trực tiếp của trục Thần kinh – Nội tiết. Khám phá cách Estradiol điều phối nồng độ Serotonin và Dopamine, cùng nguyên nhân tại sao sự sụt giảm đột ngột của Allopregnanolone trước kỳ kinh lại kích hoạt cảm giác lo âu và giảm động lực trên biểu đồ thiết bị đeo.</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>Sự sụt giảm năng lượng trước kỳ kinh là phản ứng thần kinh - hóa sinh thực tế. Lên lịch đàm phán, sáng tạo vào tuần Estrogen cao và dành tuần trước kỳ kinh cho công việc tĩnh, giảm áp lực xã hội.</t>
+          <t>Sự sụt giảm năng lượng và tính nhạy cảm cảm xúc trước kỳ kinh là phản ứng thần kinh - hóa sinh thực tế. Hãy sắp xếp các công việc đòi hỏi tư duy sáng tạo, đàm phán vào tuần Estrogen cao (ngày 6–13), và chủ động giảm tải xã hội, tăng cường giấc ngủ phục hồi trong 7 ngày trước kỳ kinh.</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1838,12 +1838,12 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>PMS vs. PMDD: Clinical Diagnostic Criteria, Brain Sensitivity &amp; Action Plan</t>
+          <t>PMS, Cramps, and Luteal Cravings: The Neuro-Endocrine Science &amp; Targeted Nutrition Protocol</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Phân Biệt PMS &amp; PMDD: Khi Căng Thẳng Tiền Kinh Nguyệt Trở Thành Hội Chứng Lâm Sàng</t>
+          <t>Hội Chứng Tiền Kinh Nguyệt (PMS), Đau Bụng Kinh &amp; Cơn Thèm Ăn Pha Hoàng Thể: Khoa Học Thần Kinh – Nội Tiết Và Phác Đồ Dinh Dưỡng</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -1908,12 +1908,12 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>Khác với nam giới vốn phụ thuộc chủ yếu vào testosterone, ham muốn ở phụ nữ là sự cộng hưởng giữa đỉnh Estradiol, testosterone tự do, oxytocin và đặc biệt là trạng thái an toàn của hệ thần kinh phó giao cảm.</t>
+          <t>Khác với nam giới vốn có cơ chế ham muốn mang tính bộc phát và phụ thuộc chủ yếu vào testosterone, ham muốn ở phụ nữ là một hệ thống phản ứng sinh học đa tầng phức tạp. Khám phá Mô hình Kiểm soát Kép (Dual Control Model), vai trò của oxytocin và lý do vì sao chỉ số HRV cao trên đồng hồ là điều kiện tiên quyết cho sự thăng hoa phòng the.</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Hưng phấn nữ giới đòi hỏi sự thư giãn giao cảm (HRV cao). Bất kỳ tình trạng kiệt sức, thiếu ngủ hay áp lực công việc nào cũng sẽ đóng sập cánh cửa ham muốn trước khi hormone kịp phát huy tác dụng.</t>
+          <t>Hưng phấn ở phụ nữ vận hành theo cơ chế 'nhả chân phanh' (hạ cortisol, tăng HRV phó giao cảm) trước khi có thể 'nhấn chân ga' (kích hoạt dopamine và oxytocin). Bất kỳ tình trạng căng thẳng mãn tính hay kiệt sức nào cũng sẽ tự động kích hoạt hệ thống ức chế tình dục (SIS) của não bộ.</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -1968,12 +1968,12 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Trong 24-48 giờ trước rụng trứng, đỉnh Estradiol kết hợp đợt tăng vọt testosterone ngắn hạn thúc đẩy ham muốn sinh học đạt đỉnh; sang pha hoàng thể, progesterone tăng cao chuyển hướng năng lượng sang trạng thái bảo vệ tổ ấm.</t>
+          <t>Nghiên cứu sinh hóa hormone của Roney &amp; Simmons (2013) khẳng định ham muốn tình dục ở nữ giới dao động có quy luật toán học theo từng ngày của chu kỳ kinh nguyệt. Khám phá lý do tại sao tự nhiên lại lập trình đỉnh hưng phấn vào cửa sổ thụ thai, và cách progesterone đưa cơ thể về trạng thái bảo tồn năng lượng trong pha hoàng thể.</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>Hiểu được đường cong ham muốn tự nhiên giúp các cặp đôi đồng điệu cảm xúc, xóa bỏ tự ti và tận dụng cửa sổ rụng trứng (ngày 12-15) cho đời sống gối chăn thăng hoa nhất.</t>
+          <t>Đỉnh ham muốn tự nhiên của bạn xuất hiện vào các ngày 11–15 của chu kỳ (khi estrogen và testosterone chạm đỉnh), trong khi sự suy giảm ham muốn ở pha hoàng thể là phản ứng sinh tồn để nuôi dưỡng tổ ấm. Hãy đồng bộ hóa đời sống lứa đôi theo nhịp sinh học này để giải phóng bản thân khỏi áp lực.</t>
         </is>
       </c>
       <c r="K14" s="7" t="inlineStr">
@@ -2028,12 +2028,12 @@
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>Âm đạo khỏe mạnh được thống trị bởi vi khuẩn Lactobacillus tiết ra axit lactic, duy trì độ pH lý tưởng 3.8–4.5. Sự suy giảm estrogen sau kỳ kinh hoặc thói quen thụt rửa làm xáo trộn hệ đệm này, dẫn đến viêm nhiễm BV và nấm ngứa.</t>
+          <t>Âm đạo là một hệ sinh thái tự làm sạch tinh vi được bảo vệ bởi hàng tỷ vi khuẩn Lactobacillus. Hiểu rõ sự tương tác giữa estrogen, glycogen và độ pH từ 3.8 đến 4.5 giúp bạn dễ dàng phân biệt dịch tiết sinh lý bình thường theo chu kỳ với các dấu hiệu cảnh báo viêm nhiễm cần can thiệp y khoa.</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>Dịch tiết trong, trắng sữa không mùi hoặc hơi chua nhẹ là hoàn toàn bình thường. Không dùng xà phòng kiềm thụt rửa; ưu tiên đồ lót cotton thoáng khí và bổ sung men vi sinh Lactobacillus rhamnosus GR-1.</t>
+          <t>Khí hư thay đổi từ lỏng trong suốt sang đục dính là hoàn toàn sinh lý theo dao động estrogen. Hãy bảo tồn lớp vi sinh vật tự nhiên bằng cách kiêng tuyệt đối thụt rửa sâu, chọn quần lót cotton thoáng khí và theo dõi triệu chứng mùi hôi hoặc ngứa rát song hành cùng pha chu kỳ trên ứng dụng.</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2088,12 +2088,12 @@
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>Đau khi quan hệ tình dục ảnh hưởng tới 10-20% phụ nữ, bắt nguồn từ sàn chậu co cứng (hypertonic pelvic floor), thiếu hụt estrogen gây khô teo mô niêm mạc, hoặc bệnh lý tiềm ẩn như lạc nội mạc tử cung.</t>
+          <t>Đau rát khi quan hệ tình dục không bao giờ là điều bạn phải cắn răng chịu đựng hay xem là chuyện 'bình thường'. Từ sự co thắt quá mức của các bó cơ sàn chậu đến tình trạng suy giảm estrogen hay lạc nội mạc tử cung, y học hiện đại có các phác đồ chuẩn xác để chữa lành tận gốc chứng giao hợp đau (Dyspareunia).</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>Đau khi quan hệ không bao giờ là điều phải cắn răng chịu đựng. Vật lý trị liệu giãn sàn chậu, bổ sung chất bôi trơn gốc nước có độ pH 3.8-4.2 và kiểm tra phụ khoa giúp phục hồi 85% trường hợp.</t>
+          <t>Nếu bạn bị đau rát khi quan hệ, giải pháp đầu tiên không phải là 'cố gắng chịu đựng' hay tập Kegel siết chặt cơ. Hãy phân biệt đau nông tại cửa mình (cần khám nơ-ron tiền đình, phục hồi màng nhầy) hay đau sâu trong ổ bụng (cần tầm soát lạc nội mạc, nang buồng trứng), đồng thời ưu tiên các bài tập hạ trương lực cơ sàn chậu.</t>
         </is>
       </c>
       <c r="K16" s="7" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>The Female Pelvic Floor Engine: Continence, Core Stability &amp; Vitality</t>
+          <t>The Female Pelvic Floor Engine: Continence, Core Stability &amp; Sexual Vitality</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -2148,12 +2148,12 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>Sàn chậu nữ nâng đỡ bàng quang, tử cung và trực tràng trước áp lực ổ bụng. Quá trình mang thai, sinh nở hoặc ngồi nhiều làm suy yếu cơ nâng hậu môn, dẫn đến són tiểu khi hắt hơi (SUI) và giảm độ nhạy tình dục.</t>
+          <t>Sàn chậu không chỉ liên quan đến câu chuyện tiểu són hay sinh nở—đây là nền tảng cơ học nâng đỡ toàn bộ nội tạng, tạo lực bộc phát trong từng bước chạy và điều phối cực khoái trong đời sống lứa đôi. Khám phá cách vận hành 'chiếc hộp áp lực ổ bụng' và lý do tại sao tập siết cơ không đúng cách có thể phản tác dụng.</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>Tập Kegel nữ chuẩn xác đòi hỏi cả pha nâng (lift) và pha thả lỏng hoàn toàn (relax). Tuyệt đối không siết mông hay nín thở; kết hợp thở cơ hoành để kích hoạt phối hợp sàn chậu - cơ hoành - cơ ngang bụng.</t>
+          <t>Sàn chậu khỏe mạnh không phải là sàn chậu luôn siết chặt, mà là sàn chậu có khả năng co giãn linh hoạt theo từng nhịp thở. Hãy kết hợp thở cơ hoành (Piston Breathing) trong từng rep tập kháng lực và lắng nghe các tín hiệu rò rỉ tiểu hoặc tức nặng vùng chậu trên ứng dụng để điều chỉnh áp lực kịp thời.</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2198,12 +2198,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Cycle-Synced Training: Harnessing High-Estrogen PRs &amp; High-Progesterone Recovery</t>
+          <t>Cycle-Synced Training: How to Periodize Strength, HIIT, and Recovery Across Your Menstrual Cycle</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Tập Luyện Đồng Bộ Chu Kỳ: Cách Tận Dụng Sức Mạnh Estrogen &amp; Phục Hồi Ở Pha Hoàng Thể</t>
+          <t>Tập Luyện Đồng Bộ Chu Kỳ (Cycle-Synced Training): Cách Phân Kỳ Sức Mạnh, HIIT Và Phục Hồi Theo Nội Tiết Tố</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -2268,12 +2268,12 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>Tập thể dục nhẹ nhàng trong ngày đèn đỏ giúp kích thích giải phóng endorphin tự nhiên, làm giãn cơ tử cung và giảm đau bụng kinh. Tuy nhiên, tránh các tư thế dốc ngược lâu và giảm tải tạ nặng vào Ngày 1–2.</t>
+          <t>Nhiều phụ nữ phân vân liệu có nên tập luyện khi đang có kinh hay nên nằm yên nghỉ ngơi hoàn toàn. Khoa học thể thao chứng minh vận động cường độ nhẹ đến vừa kích hoạt giải phóng Endorphin giảm đau tự nhiên và tăng cường lưu thông máu vùng chậu. Khám phá cách điều chỉnh tải trọng (Deload) chuẩn xác theo tín hiệu thiết bị đeo.</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>Đi bộ nhanh Zone 1, yoga phục hồi hoặc bơi nhẹ giúp giảm đau bụng kinh hiệu quả hơn nằm yên. Khi cảm thấy mệt mỏi do thiếu máu nhẹ, hãy xem đây là tuần deload tự nhiên để cơ thể chuẩn bị bứt phá.</t>
+          <t>Bạn không cần ngừng tập khi có kinh, nhưng hãy hạ cường độ từ ngưỡng bộc phát (RPE 8–10) xuống mức kích thích phục hồi (RPE 5–6) trong 48 giờ đầu. Ưu tiên đi bộ nhanh, yoga giãn mạc hoặc bơi nhẹ để hạ nồng độ prostaglandin gây co thắt tử cung.</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr">
@@ -2328,12 +2328,12 @@
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>Nghiên cứu trên thiết bị đeo ghi nhận chỉ số HRV RMSSD ở nữ đạt đỉnh ở nửa cuối pha nang trứng, sau đó sụt giảm 5-15% trong suốt pha hoàng thể do progesterone kích thích trung tâm giao cảm.</t>
+          <t>Nếu bạn nhận thấy điểm Biến thiên nhịp tim (HRV) của mình đột ngột sụt giảm 10–15% và điểm Phục hồi chuyển sang màu vàng trong hai tuần cuối của tháng, đừng hoảng sợ rằng bạn bị kiệt sức. Đó là một hiện tượng sinh lý học bình thường do progesterone chi phối hệ thần kinh thực vật.</t>
         </is>
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>HRV giảm vào tuần trước kỳ kinh là phản ứng sinh lý lành mạnh của progesterone—không phải dấu hiệu bạn bị quá tải tập luyện. Hãy so sánh HRV của bạn với đường nền theo từng pha chứ không dùng đường nền cố định.</t>
+          <t>Đừng so sánh chỉ số HRV pha hoàng thể với pha nang trứng. Hãy xây dựng hai đường cơ sở (Baseline) riêng biệt cho cơ thể: một mức nền cao ở nửa đầu chu kỳ (nhờ estrogen kích hoạt hệ phó giao cảm) và một mức nền thấp hơn ở nửa sau chu kỳ (do progesterone kích hoạt hệ giao cảm và tăng nhiệt độ cơ thể).</t>
         </is>
       </c>
       <c r="K20" s="7" t="inlineStr">
@@ -2388,12 +2388,12 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>Phụ nữ mất tới 20% mật độ xương trong 5 năm đầu sau mãn kinh do estrogen suy giảm. Nâng tạ và tập kháng lực là kích thích cơ học duy nhất ép xương kích hoạt tạo cốt bào (osteoblasts) và duy trì cơ bắp.</t>
+          <t>Tập tạ không khiến phụ nữ bị 'đô con' hay thô kệch—đó là tấm khiên y khoa vững chắc nhất để bảo vệ mật độ xương trước nguy cơ loãng xương, tối ưu hóa độ nhạy insulin và duy trì tốc độ chuyển hóa cơ bản suốt cuộc đời. Khám phá khoa học đằng sau các bài tập tạ nặng và thử nghiệm lâm sàng LIFTMOR.</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>Tập các bài compound (Squat, Deadlift, Hip Thrust, Overhead Press) 2-3 buổi/tuần không hề làm nữ giới "đô con" mà giúp eo thon, tăng độ nhạy insulin và bảo vệ xương khớp suốt đời.</t>
+          <t>Phụ nữ đạt đỉnh mật độ xương ở tuổi 25–30 và mất xương nhanh chóng sau mãn kinh. Các bài tập cardio nhẹ không đủ lực kích hoạt tế bào tạo xương; bạn cần các bài tập kháng lực đa khớp (Squat, Deadlift, Overhead Press) với mức tạ từ 70–85% 1RM ít nhất 2–3 lần mỗi tuần.</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
@@ -2448,12 +2448,12 @@
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>Khi năng lượng nạp vào không đủ bù đắp năng lượng tiêu hao cho tập luyện (&lt;30 kcal/kg FFM/ngày), cơ thể sẽ tắt chức năng sinh sản (mất kinh FHA), làm lao dốc nồng độ estrogen, giảm mật độ xương và tăng vọt nguy cơ chấn thương.</t>
+          <t>Mất kinh không phải là 'huy chương danh dự' chứng minh bạn tập luyện chăm chỉ hay giảm mỡ thành công; đó là hồi chuông báo động đỏ của cơ thể khi rơi vào Hội chứng Thiếu Hụt Năng Lượng Tương Đối Trong Thể Thao (RED-S). Tìm hiểu công thức tính năng lượng sẵn có và cách cứu vãn buồng trứng cùng khung xương trước khi quá muộn.</t>
         </is>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>Mất kinh khi tập nặng không phải "thành tích"—đó là tiếng kêu cứu sinh học của cơ thể. Nếu chu kỳ biến mất trên 3 tháng kèm HRV thấp liên tục, cần tăng calo nạp vào ngay, đặc biệt là carbohydrate.</t>
+          <t>Nếu chu kỳ kinh nguyệt của bạn bị trễ trên 35 ngày hoặc biến mất hoàn toàn kết hợp với tập luyện nặng và ăn kiêng gắt gao, bạn đang bị thiếu năng lượng sẵn có (&lt; 30 kcal/kg FFM/ngày). Hãy ngừng ngay việc cắt giảm tinh bột, giảm bớt tải trọng tập luyện (Strain) và theo dõi sự phục hồi của thân nhiệt cùng HRV trên ứng dụng.</t>
         </is>
       </c>
       <c r="K22" s="7" t="inlineStr">
@@ -2508,12 +2508,12 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>Progesterone làm tăng nhiệt độ cơ thể lõi thêm 0.3-0.5°C ở pha hoàng thể, ngăn cản cơ chế hạ nhiệt tự nhiên cần thiết để chìm vào giấc ngủ sâu. Đồng thời, cấu trúc giấc ngủ ghi nhận tỷ lệ thức giấc giữa đêm tăng và REM giảm.</t>
+          <t>Nếu bạn thường xuyên trằn trọc, đổ mồ hôi đêm hoặc tỉnh giấc giữa chừng vào tuần lễ trước kỳ kinh, đó không phải là sự trùng hợp ngẫu nhiên. Sự gia tăng nồng độ progesterone đẩy thân nhiệt cơ bản lên cao, làm xáo trộn cơ chế làm mát tự nhiên của não bộ và cắt vụn các chu kỳ ngủ sâu.</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>Hạ nhiệt độ phòng ngủ xuống 18°C (65°F), tắm nước ấm 90 phút trước ngủ để kích hoạt giãn mạch ngoại vi, và bổ sung Magie glycinate (300-400 mg) trong 10 ngày trước kỳ kinh để bảo vệ giấc ngủ.</t>
+          <t>Để đi vào giấc ngủ sâu, nhiệt độ cơ thể cần hạ xuống khoảng 1°C. Ở pha hoàng thể, progesterone ngăn chặn bước hạ nhiệt này. Hãy chủ động làm mát cơ thể: hạ điều hòa phòng ngủ xuống 18°C–19°C, tắm nước ấm trước khi ngủ 90 phút để kích thích giãn mạch ngoại vi, và hạn chế ăn khuya.</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -2568,12 +2568,12 @@
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>Khi stress kéo dài, trục HPA bơm cortisol và CRH vào máu, trực tiếp ức chế xung tiết GnRH từ vùng dưới đồi. Không có GnRH, tuyến yên không thể phóng thích đỉnh LH, khiến nang trứng không rụng và chu kỳ bị kéo dài.</t>
+          <t>Một kỳ thi căng thẳng, một dự án áp lực cao hoặc cú sốc tinh thần có thể khiến kỳ kinh của bạn biến mất cả tháng. Đó không phải là lỗi của buồng trứng, mà là cơ chế sinh tồn ưu việt của não bộ: khi trục HPA phát tín hiệu nguy hiểm, vùng hạ đồi sẽ lập tức hoãn việc rụng trứng để bảo vệ bạn khỏi việc mang thai trong hoàn cảnh ngặt nghèo.</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>Một kỳ kinh trễ 1-2 tuần sau đợt deadline căng thẳng là phản ứng sinh tồn tự nhiên nhằm bảo vệ bạn khỏi việc mang thai trong môi trường bất an. Ưu tiên thở 5.5 giây và ngủ đủ giấc để tái lập nhịp HPO.</t>
+          <t>Khi gặp căng thẳng nặng, trứng không thể rụng đúng hạn khiến chu kỳ bị kéo dài. Đừng uống thuốc ép kinh bừa bãi. Hãy theo dõi điểm Căng thẳng Thần kinh (Stress Monitor) và HRV trên thiết bị đeo; khi nhịp tim nghỉ ngơi hạ nhiệt và hệ phó giao cảm hồi phục, buồng trứng sẽ tự động kích hoạt rụng trứng trở lại.</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr">
@@ -2628,12 +2628,12 @@
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>Pha nang trứng tối ưu cho việc đốt và dự trữ glycogen nhờ độ nhạy insulin cao từ estrogen. Sang pha hoàng thể, tốc độ trao đổi chất cơ bản tăng 100-250 kcal/ngày, tăng dị hóa protein và tăng phân giải mỡ.</t>
+          <t>Cơ thể phụ nữ không phải là một cỗ máy chuyển hóa bất biến như nam giới; khả năng đốt mỡ, dung nạp tinh bột và phân hủy protein thay đổi rõ rệt qua từng tuần theo nồng độ hormone. Áp dụng dinh dưỡng đồng bộ chu kỳ (Cycle-Synced Nutrition) giúp bạn đập tan cơn thèm đồ ngọt tiền kinh nguyệt và tối ưu hiệu suất thể thao.</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>Nạp tinh bột phức hợp và tập cường độ cao ở tuần 1–2; tăng lượng protein (1.6-2.0 g/kg), bổ sung chất béo lành mạnh và ăn nhẹ trước tập ở tuần 3–4 để ngăn chặn dị hóa cơ bắp.</t>
+          <t>Tận dụng độ nhạy insulin cao ở nửa đầu chu kỳ (Pha Nang trứng) để nạp tinh bột phức hợp phục vụ các bài tập nặng. Ở nửa sau chu kỳ (Pha Hoàng thể), khi tốc độ chuyển hóa cơ bản tăng 100–250 kcal/ngày nhưng cơ thể dễ bị dị hóa cơ bắp, hãy tăng lượng protein lên 1.8–2.0g/kg và bổ sung chất béo lành mạnh.</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
@@ -2688,12 +2688,12 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>Mất hơn 80 ml máu mỗi kỳ kinh (Menorrhagia) làm cạn kiệt kho dự trữ sắt Ferritin mà xét nghiệm huyết sắc tố thông thường có thể bỏ sót, gây mệt mỏi mạn tính, hụt hơi khi leo cầu thang và sụt giảm VO2 Max.</t>
+          <t>Bạn cảm thấy tim đập thình thịch khi leo cầu thang, hụt hơi khi chạy bộ dù kết quả xét nghiệm máu cho thấy nồng độ Hemoglobin 'bình thường'? Rất có thể bạn đang bị thiếu sắt tiềm ẩn (Tụt Ferritin) do kinh nguyệt ra nhiều (Menorrhagia). Khám phá cách chẩn đoán và phác đồ bù sắt chuẩn y học thể thao.</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>Nếu phải thay băng vệ sinh mỗi 1-2 giờ hoặc có cục máu đông lớn hơn đồng xu, hãy yêu cầu xét nghiệm Ferritin huyết thanh (ngưỡng tối ưu &gt;50 ng/mL). Bổ sung sắt kèm vitamin C vào buổi sáng cách xa cà phê.</t>
+          <t>Đừng chỉ kiểm tra nồng độ Hemoglobin; hãy yêu cầu bác sĩ xét nghiệm Ferritin huyết thanh (mục tiêu tối ưu cho phụ nữ vận động là &gt; 50 ng/mL). Nếu bạn phải thay băng vệ sinh sau mỗi 1–2 giờ hoặc có cục máu đông lớn hơn đồng xu, hãy bổ sung sắt hữu cơ dạng Sắt Bisglycinate uống cách ngày kết hợp cùng Vitamin C.</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
@@ -2748,12 +2748,12 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>Trong khi trứng chỉ sống được 12–24 giờ sau khi rụng, tinh trùng có thể tồn tại tới 5 ngày bên trong chất nhầy cổ tử cung màu mỡ. Do đó, cơ hội thụ thai cao nhất thực chất nằm ở 2 ngày TRƯỚC rụng trứng.</t>
+          <t>Nhiều cặp đôi lầm tưởng rằng chỉ có thể thụ thai vào đúng ngày rụng trứng, dẫn đến việc bỏ lỡ những thời điểm vàng quý giá nhất. Khám phá bí mật tuổi thọ giao tử, hiện tượng biến đổi tinh trùng (Capacitation) và cách công nghệ thiết bị đeo giúp bạn xác định chuẩn xác cửa sổ sinh sản 6 ngày.</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>Quan hệ vào các ngày −2, −1 và ngày rụng trứng mang lại xác suất thụ thai trên 85%. Không chờ đến khi nhiệt độ cơ bản tăng mới quan hệ—bởi vì khi nhiệt độ tăng, trứng đã thoái hóa.</t>
+          <t>Trứng chỉ sống được 12–24 giờ sau khi rụng, nhưng tinh trùng có thể sống khỏe mạnh tới 3–5 ngày trong dịch nhầy cổ tử cung giàu estrogen. Để tối đa hóa cơ hội có thai, hãy quan hệ vào 1–2 ngày TRƯỚC KHI rụng trứng thay vì chờ đến khi nhiệt độ cơ thể đã tăng vọt.</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -2808,12 +2808,12 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>Sau khi phôi nang làm tổ vào ngày 8–10 sau rụng trứng, hormone hCG duy trì hoàng thể tiếp tục tiết progesterone. Trên thiết bị đeo, nhiệt độ da ban đêm neo cao liên tục trên 18 ngày là chỉ dấu thụ thai sớm.</t>
+          <t>Trước khi que thử thai xuất hiện 2 vạch rõ ràng, cơ thể bạn đã âm thầm diễn ra một cuộc cách mạng sinh học vi mô. Khi phôi nang làm tổ thành công vào nội mạc tử cung, các thuật toán trên thiết bị đeo thông minh có thể phát hiện bước nhảy thân nhiệt thứ ba (Triphasic BBT) và sự gia tăng nhịp tim nghỉ ngơi từ nhiều ngày trước kỳ kinh dự kiến.</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>Đường cong nhiệt độ 3 pha (Triphasic curve) và nhịp tim nghỉ ngơi (RHR) bắt đầu tăng dần 1-2 nhịp/phút ngay từ tuần thai thứ 4 là những tín hiệu sinh lý sớm nhất trước cả khi que thử thai hiện rõ 2 vạch.</t>
+          <t>Dấu hiệu mang thai sớm nhất trên thiết bị đeo là biểu đồ nhiệt độ 3 pha (Triphasic pattern): nhiệt độ da ban đêm tiếp tục tăng bước nhảy thứ hai sau ngày 8–10 sau rụng trứng (DPO) thay vì hạ nhiệt chuẩn bị hành kinh, đi kèm nhịp tim nghỉ ngơi RHR tăng thêm 2–4 bpm và không có máu kinh xuất hiện.</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
@@ -2868,12 +2868,12 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>Thể tích máu tăng 40–50% và cung lượng tim tăng 30–50% để nuôi dưỡng thai nhi. Dữ liệu từ hàng nghìn thai kỳ trên WHOOP (Rowan 2022) cho thấy RHR tăng đỉnh điểm vào tuần 30 và HRV giảm liên tục.</t>
+          <t>Mang thai tương đương với việc chạy một cuộc thi marathon kéo dài 40 tuần liên tục: thể tích máu tăng 50%, tim phải đập thêm 15.000 nhịp mỗi ngày và hệ thống mạch máu tái cấu trúc toàn diện. Tìm hiểu các biến đổi sinh học phi thường qua từng tam cá nguyệt từ công trình nghiên cứu thai kỳ liên tục của WHOOP.</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>Sự sụt giảm điểm phục hồi (Recovery) và tăng nhịp tim khi mang thai là sự thích nghi tim mạch phi thường để cấp máu cho thai nhi—chứ không phải bạn bị suy kiệt thể lực. Lắng nghe cơ thể và ưu tiên nghỉ ngơi.</t>
+          <t>Nhịp tim nghỉ ngơi tăng thêm 10–15 bpm và điểm HRV sụt giảm sâu trong thai kỳ là sự thích nghi tim mạch hoàn toàn bình thường để nuôi dưỡng thai nhi, không phải dấu hiệu kiệt sức. Nhịp tim đạt đỉnh quanh tuần thứ 30 và bắt đầu ổn định chuẩn bị cho cuộc chuyển dạ.</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -2928,12 +2928,12 @@
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>Tập thể dục 150 phút/tuần ở cường độ vừa phải giúp giảm 50% nguy cơ tiểu đường thai kỳ và tiền sản giật theo Hiệp hội Sản Phụ khoa Hoa Kỳ (ACOG). Tránh nằm ngửa sau tam cá nguyệt 1 và tránh bài tập gây va đập.</t>
+          <t>Quan niệm cổ hủ cho rằng phụ nữ mang thai phải nằm yên dưỡng thai đã bị y học hiện đại bác bỏ hoàn toàn. Tập luyện đúng cách trong thai kỳ giúp giảm 50% nguy cơ tiểu đường thai kỳ, hạ tỷ lệ sinh mổ và bảo vệ vùng thắt lưng. Khám phá hướng dẫn an toàn chuẩn mực từ Đại học Sản Phụ khoa Hoa Kỳ (ACOG).</t>
         </is>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>Sử dụng bài kiểm tra trò chuyện (Talk Test) hoặc giữ nhịp tim trong vùng Zone 2–3 hiếu khí. Đi bộ, bơi lội, đạp xe cố định và tập tạ nhẹ với tư thế bảo vệ sàn chậu là những lựa chọn an toàn tuyệt đối.</t>
+          <t>Phụ nữ mang thai không có biến chứng nên duy trì ít nhất 150 phút vận động cường độ vừa phải mỗi tuần. Sử dụng 'Bài kiểm tra nói chuyện' (Talk Test) hoặc giữ nhịp tim dưới 60%–70% nhịp tim tối đa; tránh tuyệt đối các bài tập nằm ngửa sau tuần 16, các môn thể thao va chạm mạnh và các môi trường quá nóng.</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
@@ -2988,12 +2988,12 @@
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>Sau sinh, hormone relaxin vẫn duy trì độ giãn dây chằng trong nhiều tháng, cơ bụng bị kéo giãn dọc đường trắng (linea alba) và sàn chậu cần thời gian lành mô. Đồng thời, chỉ số HRV bật tăng trở lại ngay tuần đầu sau sinh.</t>
+          <t>Hành trình làm mẹ không dừng lại ở phòng sinh; 12 tuần đầu tiên sau khi sinh—được y học gọi là 'Tam Cá Nguyệt Thứ Tư'—là giai đoạn cơ thể trải qua cú sốc tụt dốc hormone lớn nhất đời người cùng sự tái cấu trúc cơ bụng và sàn chậu. Khám phá cách chẩn đoán tách cơ bụng (Diastasis Recti) và phác đồ phục hồi thể lực an toàn.</t>
         </is>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>Tuyệt đối không gập bụng (sit-ups) ngay vì sẽ làm rách rộng khe tách cơ bụng. Bắt đầu với bài thở kết nối cơ hoành và sàn chậu từ tuần 2; chỉ trở lại chạy bộ hoặc tạ nặng sau 12 tuần và có đánh giá chuyên gia.</t>
+          <t>Đừng vội vàng gập bụng truyền thống (Crunches/Sit-ups) sau sinh vì chúng làm tăng áp lực ổ bụng và khiến vết tách cơ bụng hở rộng hơn. Hãy bắt đầu bằng các bài tập kích hoạt cơ ngang bụng sâu (Transversus Abdominis) qua nhịp thở cơ hoành, và cho phép hệ thần kinh 1–2 tuần để nhịp tim nghỉ ngơi hạ nhiệt tự nhiên.</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -3048,12 +3048,12 @@
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>PCOS ảnh hưởng tới 10-13% phụ nữ, được chẩn đoán khi có ít nhất 2 trong 3 tiêu chuẩn Rotterdam. Bản chất sâu xa của 70% ca PCOS là tình trạng kháng insulin, kích thích buồng trứng sản xuất thừa androgen.</t>
+          <t>PCOS không đơn thuần là sự xuất hiện của các nang nhỏ trên buồng trứng; đó là một hội chứng rối loạn chuyển hóa và nội tiết toàn thân phức tạp ảnh hưởng đến 1 trên 10 phụ nữ. Tìm hiểu tiêu chuẩn chẩn đoán Rotterdam quốc tế, vai trò cốt lõi của tình trạng kháng insulin và phác đồ tập luyện dinh dưỡng để phục hồi chu kỳ rụng trứng.</t>
         </is>
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>Chìa khóa quản lý PCOS không phải ăn kiêng cực đoan mà là cải thiện độ nhạy insulin: đi bộ 10 phút sau ăn, tập tạ kháng lực 3 buổi/tuần, bổ sung Inositol (tỷ lệ 40:1 Myo/D-chiro) và ngủ đủ giấc.</t>
+          <t>Để chẩn đoán PCOS chuẩn xác, bạn cần thỏa mãn ít nhất 2 trong 3 tiêu chuẩn Rotterdam: kinh nguyệt thưa/vô kinh, dấu hiệu thừa androgen (rậm lông, mụn bọc, rụng tóc), hoặc hình ảnh đa nang trên siêu âm. Chìa khóa điều trị số 1 không phải là thuốc tránh thai mà là giải quyết tình trạng Kháng Insulin bằng tập tạ kháng lực và bổ sung Myo-Inositol.</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
@@ -3108,12 +3108,12 @@
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>Khi các mô tương tự niêm mạc tử cung phát triển bên ngoài buồng tử cung (buồng trứng, phúc mạc), chúng chảy máu theo chu kỳ nhưng không có đường thoát, gây viêm mạn tính, dính mô và đau dữ dội.</t>
+          <t>Đau bụng kinh dữ dội đến mức ngất xỉu, nôn mửa hoặc phải nghỉ làm không bao giờ là chuyện 'bình thường'. Lạc nội mạc tử cung (Endometriosis) là một bệnh lý viêm mãn tính phức tạp hành hạ gần 200 triệu phụ nữ trên toàn cầu, với độ trễ chẩn đoán trung bình từ 7 đến 10 năm. Tìm hiểu cơ chế sinh học, dấu hiệu cảnh báo và lộ trình điều trị y khoa chuẩn mực.</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>Đau bụng kinh dữ dội không đỡ sau khi uống thuốc giảm đau, đau khi đại tiện hoặc quan hệ là dấu hiệu điển hình của lạc nội mạc tử cung. Chẩn đoán sớm giúp bảo tồn buồng trứng và chất lượng cuộc sống.</t>
+          <t>Nếu cơn đau bụng kinh của bạn không thuyên giảm khi dùng thuốc giảm đau NSAIDs thông thường, hoặc lan ra sau lưng, đau buốt khi đi vệ sinh hay khi quan hệ sâu, đừng chần chừ. Hãy tìm đến bác sĩ chuyên khoa sâu về Lạc nội mạc tử cung để siêu âm chuyên sâu hoặc phẫu thuật nội soi bóc tách tổn thương.</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -3168,12 +3168,12 @@
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>Trong giai đoạn tiền mãn kinh (bắt đầu từ tuổi 40-45), nồng độ estrogen trồi sụt dữ dội trước khi giảm hẳn, làm xáo trộn trung tâm điều nhiệt gây bốc hỏa ban đêm và đẩy nhịp tim nghỉ ngơi tăng cao.</t>
+          <t>Thời kỳ tiền mãn kinh không phải là một công tắc bật tắt đột ngột ở tuổi 50; đó là một giai đoạn chuyển tiếp nội tiết kéo dài từ 4 đến 8 năm, bắt đầu từ độ tuổi ngoài 40 với những đợt sóng estrogen dao động dữ dội. Tìm hiểu tiêu chuẩn vàng STRAW+10, nguồn gốc các cơn bốc hỏa và chiến lược y học hiện đại để bước qua giai đoạn này với sức sống rạng ngời.</t>
         </is>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>Bảo tồn mật độ xương bằng tập tạ nặng và bổ sung Canxi + Vitamin D3/K2; theo dõi nhiệt độ da ban đêm để nhận diện cơn bốc hỏa và thảo luận với bác sĩ về liệu pháp hormone mãn kinh (MHT).</t>
+          <t>Mãn kinh chỉ được xác định khi bạn đã mất kinh liên tục trọn vẹn 12 tháng. Trong giai đoạn tiền mãn kinh, hãy theo dõi sự dãn dài của chu kỳ (&gt; 7 ngày lệch chuẩn) trên thiết bị đeo, chủ động rèn luyện tạ kháng lực để chống mất xương và thảo luận sớm với bác sĩ về Liệu Pháp Hormone Mãn Kinh (MHT) trong 'Cửa Sổ Vàng' trước tuổi 60.</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(content): audit health guidance, references, illustrations and workbook exports
</commit_message>
<xml_diff>
--- a/docs/Master_Health_Articles_MVP - 30 Blog Topics.xlsx
+++ b/docs/Master_Health_Articles_MVP - 30 Blog Topics.xlsx
@@ -7,8 +7,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master_Health_Articles_MVP - 30" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewed_Content" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Register" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Reviewed_Content'!$A$1:$H$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source_Register'!$A$1:$F$36</definedName>
+  </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -192,8 +197,16 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill/>
     </fill>
@@ -398,6 +411,11 @@
         <bgColor rgb="00ECFDF5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00184E52"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -669,7 +687,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -694,6 +712,15 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1295,7 +1322,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L34"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.4375" defaultRowHeight="16.8" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.4375" defaultRowHeight="16.8"/>
   <cols>
     <col width="8" customWidth="1" style="1" min="1" max="1"/>
     <col width="24" customWidth="1" style="1" min="2" max="2"/>
@@ -1398,7 +1425,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Understanding Your Menstrual Cycle</t>
+          <t>Understanding menstrual cycle phases</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1408,7 +1435,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Completed (Mapped to LM_WH_01)</t>
+          <t>Revised — LM_WH_01; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -1418,32 +1445,32 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>The 4 Phases of Your Menstrual Cycle: How Hormones Shape Your Energy, Sleep, and Wearable Biometrics</t>
+          <t>Understanding menstrual cycle phases</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>4 Giai Đoạn Của Chu Kỳ Kinh Nguyệt: Cách Hormone Điều Phối Năng Lượng, Giấc Ngủ Và Chỉ Số Sinh Học Trên Thiết Bị Đeo</t>
+          <t>Chu kỳ kinh nguyệt: hiểu các giai đoạn mà không đóng khung bản thân</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Cơ thể nữ giới vận hành theo hai nhịp sinh học song hành: nhịp ngày đêm 24 giờ (Circadian) và chu kỳ nội tiết khoảng 28 ngày (Infradian). Khám phá cách sự thăng trầm của Estrogen và Progesterone làm thay đổi nhiệt độ da ban đêm, nhịp tim lúc nghỉ (RHR), biến thiên nhịp tim (HRV) và năng lượng qua 4 giai đoạn.</t>
+          <t>Chu kỳ được tính từ ngày đầu kỳ kinh này đến ngày đầu kỳ kế tiếp.</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Đừng kỳ vọng điểm Sẵn sàng (Readiness), Nhịp tim lúc nghỉ (RHR) hay sức bền của bạn giữ nguyên một đường thẳng suốt cả tháng. Ở giai đoạn Nang trứng, Estrogen tăng cao giúp nâng HRV và hạ RHR—thời điểm vàng cho các bài tập cường độ cao. Sang giai đoạn Hoàng thể, Progesterone làm tăng nhiệt độ cơ thể thêm +0.3°C đến +0.5°C và đẩy RHR tăng 3–7 bpm, báo hiệu cơ thể cần chuyển sang vận động ổn định và ưu tiên phục hồi.</t>
+          <t>Ghi ngày bắt đầu, thời lượng, mức chảy máu và triệu chứng theo cách dễ duy trì. Dùng thông tin để chuẩn bị chăm sóc bản thân và trao đổi khi khám, không dùng lịch để quyết định năng lực mỗi ngày.</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>HO-01 (Period duration), HO-02 (Cycle length median 29.3d - Bull 2019), HO-04 (4 Phases)</t>
+          <t>Understanding menstrual cycle phases (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Critchley et al. (Lancet, 2020); Bull et al. (npj Digit Med, 2019, 600k cycles); Baker et al. (2020)</t>
+          <t>https://www.nhs.uk/conditions/periods/</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1485,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>The 4 Phases of Your Cycle Explained</t>
+          <t>Understanding menstrual cycle phases</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1468,7 +1495,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Completed (Mapped to LM_WH_01)</t>
+          <t>Revised — LM_WH_01; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -1478,32 +1505,32 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>The 4 Phases of Your Menstrual Cycle: How Hormones Shape Your Energy, Sleep, and Wearable Biometrics</t>
+          <t>Understanding menstrual cycle phases</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>4 Giai Đoạn Của Chu Kỳ Kinh Nguyệt: Cách Hormone Điều Phối Năng Lượng, Giấc Ngủ Và Chỉ Số Sinh Học Trên Thiết Bị Đeo</t>
+          <t>Chu kỳ kinh nguyệt: hiểu các giai đoạn mà không đóng khung bản thân</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Cơ thể nữ giới vận hành theo hai nhịp sinh học song hành: nhịp ngày đêm 24 giờ (Circadian) và chu kỳ nội tiết khoảng 28 ngày (Infradian). Khám phá cách sự thăng trầm của Estrogen và Progesterone làm thay đổi nhiệt độ da ban đêm, nhịp tim lúc nghỉ (RHR), biến thiên nhịp tim (HRV) và năng lượng qua 4 giai đoạn.</t>
+          <t>Chu kỳ được tính từ ngày đầu kỳ kinh này đến ngày đầu kỳ kế tiếp.</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Đừng kỳ vọng điểm Sẵn sàng (Readiness), Nhịp tim lúc nghỉ (RHR) hay sức bền của bạn giữ nguyên một đường thẳng suốt cả tháng. Ở giai đoạn Nang trứng, Estrogen tăng cao giúp nâng HRV và hạ RHR—thời điểm vàng cho các bài tập cường độ cao. Sang giai đoạn Hoàng thể, Progesterone làm tăng nhiệt độ cơ thể thêm +0.3°C đến +0.5°C và đẩy RHR tăng 3–7 bpm, báo hiệu cơ thể cần chuyển sang vận động ổn định và ưu tiên phục hồi.</t>
+          <t>Ghi ngày bắt đầu, thời lượng, mức chảy máu và triệu chứng theo cách dễ duy trì. Dùng thông tin để chuẩn bị chăm sóc bản thân và trao đổi khi khám, không dùng lịch để quyết định năng lực mỗi ngày.</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>HO-04 (Estimated cycle phase: Menstrual/Follicular/Ovulatory/Luteal), appleSleepingWristTemperature</t>
+          <t>Understanding menstrual cycle phases (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>Baker et al. (2020); Sims et al. (PLOS ONE / BMJ, 2021); Oura Cycle Insights Clinical Studies</t>
+          <t>https://www.nhs.uk/conditions/periods/</t>
         </is>
       </c>
     </row>
@@ -1518,7 +1545,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Common Period Symptoms &amp; How to Manage Them</t>
+          <t>PMS, cramps and appetite changes</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1528,7 +1555,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Completed (Mapped to DM_WH_03)</t>
+          <t>Revised — DM_WH_03; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1538,32 +1565,32 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>PMS, Cramps, and Luteal Cravings: The Neuro-Endocrine Science &amp; Targeted Nutrition Protocol</t>
+          <t>PMS, cramps and appetite changes</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Hội Chứng Tiền Kinh Nguyệt (PMS), Đau Bụng Kinh &amp; Cơn Thèm Ăn Pha Hoàng Thể: Khoa Học Thần Kinh – Nội Tiết Và Phác Đồ Dinh Dưỡng</t>
+          <t>PMS, đau bụng kinh và thèm ăn: chăm sóc theo triệu chứng</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Đau bụng kinh, biến động cảm xúc, tích nước và cơn thèm đồ ngọt dữ dội trước kỳ kinh hoàn toàn không phải do 'tâm lý'—chúng được thúc đẩy bởi chất gây viêm Prostaglandin (PGF2α) tại tử cung, mức tăng trao đổi chất 100–250 kcal/ngày và sự sụt giảm Serotonin cuối pha Hoàng thể. Đây là phác đồ vi chất lâm sàng giúp làm dịu triệt để.</t>
+          <t>PMS có thể gồm thay đổi tâm trạng, khó ngủ, căng ngực và thèm ăn trước kỳ kinh.</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Hội chứng PMS và đau bụng kinh bắt nguồn từ ba cơ chế sinh hóa hoàn toàn có thể can thiệp: co thắt cơ trơn tử cung do Prostaglandin (PGF2α), sự sụt giảm chất dẫn truyền thần kinh Serotonin và GABA cuối pha Hoàng thể, cùng mức tăng chuyển hóa cơ bản (+100–250 kcal/ngày). Bổ sung Canxi (1.000–1.200 mg), Magie Glycinate (300–400 mg), Vitamin B6 (50–80 mg) và Omega-3 EPA/DHA trong pha Hoàng thể giúp giảm rõ rệt cơn đau và ổn định tâm trạng.</t>
+          <t>Ghi triệu chứng ít nhất hai chu kỳ, gồm thời điểm bắt đầu, lúc giảm và ảnh hưởng công việc. Duy trì bữa ăn cân bằng, vận động phù hợp và ngủ đủ; dùng nhật ký để trao đổi về lựa chọn điều trị nếu cần.</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>HO-06 (Hormonal symptom logs: 22 HealthKit symptom categories, abdominalCramps, bloating)</t>
+          <t>PMS, cramps and appetite changes (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>Dawood et al. (Am J Obstet Gynecol); Pierson et al. (Nat Hum Behav, 2021); Bernardi et al. (2017)</t>
+          <t>https://www.nhs.uk/conditions/pre-menstrual-syndrome/</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1605,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Irregular Periods: What's Normal and What's Not?</t>
+          <t>Irregular periods: tracking and seeking care</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -1588,7 +1615,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_04)</t>
+          <t>Revised — WH_04; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -1598,32 +1625,32 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Irregular Cycles Decoded: When Variation is Healthy vs. A Clinical Red Flag</t>
+          <t>Irregular periods: tracking and seeking care</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Kinh Nguyệt Không Đều: Nhận Diện Chu Kỳ Không Rụng Trứng &amp; Khi Nào Là Cảnh Báo Lâm Sàng?</t>
+          <t>Kinh nguyệt không đều: ghi nhận gì và khi nào đi khám?</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Nghiên cứu quy mô lớn từ hơn 600.000 chu kỳ đăng trên tạp chí npj Digital Medicine cho thấy chỉ có khoảng 13% phụ nữ có chu kỳ đúng 28 ngày chuẩn mực. Khám phá cách các thuật toán thiết bị đeo (như Apple Health và WHOOP) nhận diện chu kỳ không rụng trứng (Anovulatory), phân biệt sự dao động sinh lý tự nhiên với các dấu hiệu cảnh báo bệnh lý cần thăm khám y khoa.</t>
+          <t>Chu kỳ thay đổi có thể liên quan tuổi, tránh thai, mang thai, stress, thay đổi cân nặng hoặc bệnh lý.</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>Dao động chu kỳ trong biên độ ±2 đến 4 ngày giữa các tháng là hoàn toàn khỏe mạnh. Bạn chỉ cần thăm khám y tế khi chu kỳ ngắn hơn 21 ngày, dài hơn 35 ngày liên tục, độ dài trồi sụt trên 8–10 ngày, hoặc thiếu bước nhảy thân nhiệt cơ bản (+0.3°C) ở nửa sau chu kỳ.</t>
+          <t>Ghi ngày bắt đầu, thời gian chảy máu, triệu chứng và thuốc. Nếu có khả năng mang thai, thử thai theo hướng dẫn. Mang lịch ghi nhận khi khám để bác sĩ chọn xét nghiệm phù hợp thay vì tự mua cả bộ hormone.</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>HO-02 (Cycle length), HO-03 (Next-period prediction: frozen median &amp; anomaly alert), Bull 2019</t>
+          <t>Irregular periods: tracking and seeking care (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>Bull et al. (npj Digit Med, 2019); Li K et al. (JAMIA, 2021 - Clue); Fraser et al. (Fertil Steril, FIGO 2011)</t>
+          <t>https://www.nhs.uk/symptoms/missed-or-late-periods/</t>
         </is>
       </c>
     </row>
@@ -1638,7 +1665,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Understanding Ovulation &amp; Your Fertile Window</t>
+          <t>The fertile window and prediction uncertainty</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1648,7 +1675,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Completed (Mapped to DM_WH_02)</t>
+          <t>Revised — DM_WH_02; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1658,32 +1685,32 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>The 6-Day Fertile Window: The Exact Biological Timeline of Conception &amp; Multi-Sensor Tracking</t>
+          <t>The fertile window and prediction uncertainty</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Cửa Sổ Thụ Thai 6 Ngày: Dòng Thời Gian Sinh Học Chính Xác Của Sự Thụ Tinh &amp; Theo Dõi Đa Cảm Biến</t>
+          <t>Cửa sổ thụ thai: dùng dự đoán với mức chắc chắn phù hợp</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Trái với lầm tưởng phổ biến, ngày rụng trứng không phải là ngày duy nhất—và thậm chí không phải là ngày có xác suất cao nhất—để thụ thai. Khám phá dữ liệu lâm sàng kinh điển trên tạp chí New England Journal of Medicine về cửa sổ thụ thai 6 ngày và cách kết hợp dịch nhầy cổ tử cung, đỉnh LH cùng nhiệt độ thiết bị đeo.</t>
+          <t>Khả năng thụ thai tập trung quanh những ngày trước và sát rụng trứng vì tinh trùng có thể sống nhiều ngày, còn trứng tồn tại ngắn hơn.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Về mặt sinh học, quá trình thụ thai chỉ có thể xảy ra trong cửa sổ 6 ngày mỗi chu kỳ: 5 ngày trước khi rụng trứng cộng với 24 giờ tuổi thọ của trứng vào đúng ngày rụng trứng. Xác suất thụ thai cao nhất trong một ngày rơi vào 1 đến 2 ngày TRƯỚC khi trứng rụng (27%–33%), khi tinh trùng khỏe mạnh đã chờ sẵn tại ống dẫn trứng trước thời khắc trứng phóng thích.</t>
+          <t>Khi mong có thai, quan hệ đều trong giai đoạn nghi dễ thụ thai có thể thực tế hơn việc cố đúng một giờ. Ghi chu kỳ và thảo luận cách dùng chất nhầy hoặc xét nghiệm LH với người có chuyên môn nếu cần.</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>HO-04 (Ovulation prediction L-14, wrist temp shift), appleSleepingWristTemperature (Wang 2025)</t>
+          <t>The fertile window and prediction uncertainty (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Wilcox et al. (NEJM); Stirnemann et al. (Hum Reprod, 2013); Wang et al. (Hum Reprod, 2025)</t>
+          <t>https://www.acog.org/womens-health/faqs/fertility-awareness-based-methods-of-family-planning</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1725,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Estrogen &amp; Progesterone: How They Affect Your Body</t>
+          <t>Estrogen and progesterone: roles and tracking limits</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -1708,7 +1735,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_06)</t>
+          <t>Revised — WH_06; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -1718,32 +1745,32 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Estrogen vs. Progesterone: The Master Systemic Orchestrators of Female Health</t>
+          <t>Estrogen and progesterone: roles and tracking limits</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Estrogen &amp; Progesterone: Bản Giao Hưởng Nội Tiết Tác Động Toàn Diện Lên Tim Mạch, Xương Khớp &amp; Não Bộ</t>
+          <t>Estrogen và progesterone: vai trò và giới hạn tự theo dõi</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Estrogen và Progesterone không chỉ điều khiển niêm mạc tử cung mà còn gắn kết với hàng triệu thụ thể chuyên biệt tại mạch máu, khung xương, tế bào thần kinh và cơ bắp. Khám phá cách hai hormone quyền lực này định hình huyết áp, khả năng phục hồi thần kinh tự chủ (HRV) và tốc độ trao đổi chất của bạn qua từng tuần.</t>
+          <t>Estrogen và progesterone tham gia điều hòa chu kỳ, sinh sản và nhiều mô trong cơ thể.</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>Estrogen là hormone bảo vệ tim mạch, tăng độ đàn hồi mạch máu và thúc đẩy đồng hóa cơ bắp; trong khi Progesterone nâng nhiệt độ cơ sở lõi, tăng phân giải axit béo và kích thích hô hấp ở nửa sau chu kỳ. Đừng cố gắng duy trì cùng một giáo án dinh dưỡng và luyện tập khi tỷ lệ E2:P4 thay đổi.</t>
+          <t>Theo dõi triệu chứng bạn muốn cải thiện, ngày kinh, thuốc và mức ảnh hưởng sinh hoạt. Khi khám, hỏi xét nghiệm có thực sự cần và cần lấy ở thời điểm nào; đừng tự dùng hormone theo biểu đồ lý thuyết.</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>HO-04 (Hormone balance tracking), REC-01 (HRV modulation: E2 boosts parasympathetic, P4 boosts sympathetic)</t>
+          <t>Estrogen and progesterone: roles and tracking limits (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>Baker et al. (2020); Mendelsohn &amp; Karas (NEJM, 1999); Mauvais-Jarvis et al. (Endocr Rev, 2017)</t>
+          <t>https://www.endocrine.org/patient-engagement/endocrine-library/hormones-and-endocrine-function/reproductive-hormones</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1785,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>How Hormones Affect Your Energy and Mood</t>
+          <t>Concentration and mood around your period</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -1768,7 +1795,7 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_07)</t>
+          <t>Revised — WH_07; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1778,32 +1805,32 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>The Neuro-Endocrine Axis: Why Energy, Focus &amp; Mood Shift Across the Month</t>
+          <t>Concentration and mood around your period</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>Trục Não Bộ - Buồng Trứng: Vì Sao Trí Lực, Sự Tập Trung &amp; Cảm Xúc Biến Động Theo Từng Tuần?</t>
+          <t>Tập trung và cảm xúc quanh kỳ kinh: theo dõi trải nghiệm thực tế</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Sự thăng trầm của cảm xúc trong tháng không bắt nguồn từ sự yếu đuối tâm lý—đó là hệ quả trực tiếp của trục Thần kinh – Nội tiết. Khám phá cách Estradiol điều phối nồng độ Serotonin và Dopamine, cùng nguyên nhân tại sao sự sụt giảm đột ngột của Allopregnanolone trước kỳ kinh lại kích hoạt cảm giác lo âu và giảm động lực trên biểu đồ thiết bị đeo.</t>
+          <t>Một số người thấy khó ngủ, mệt hoặc khó tập trung trước kỳ kinh, nhưng trải nghiệm rất khác nhau.</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>Sự sụt giảm năng lượng và tính nhạy cảm cảm xúc trước kỳ kinh là phản ứng thần kinh - hóa sinh thực tế. Hãy sắp xếp các công việc đòi hỏi tư duy sáng tạo, đàm phán vào tuần Estrogen cao (ngày 6–13), và chủ động giảm tải xã hội, tăng cường giấc ngủ phục hồi trong 7 ngày trước kỳ kinh.</t>
+          <t>Trong hai chu kỳ, ghi mức tập trung, giấc ngủ và triệu chứng thay vì chỉ ngày kinh. Nếu nhận ra mẫu riêng, sắp xếp nghỉ hoặc công việc linh hoạt khi có thể. Không cần tự hạn chế nhiệm vụ vào một pha được app dự đoán.</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>HO-06 (Mood logs), HO-07 (Symptom prediction - Pierson 2021 Nature Human Behaviour), REC-03 (Stress score)</t>
+          <t>Concentration and mood around your period (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>Barth et al. (Neuropsychopharmacology, 2015); Epperson et al. (Am J Psychiatry, 2012); Pierson et al. (2021)</t>
+          <t>https://www.nhs.uk/conditions/pre-menstrual-syndrome/</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1845,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Understanding PMS &amp; PMDD</t>
+          <t>PMS, cramps and appetite changes</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1828,7 +1855,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Completed (Mapped to DM_WH_03)</t>
+          <t>Revised — DM_WH_03; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -1838,32 +1865,32 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>PMS, Cramps, and Luteal Cravings: The Neuro-Endocrine Science &amp; Targeted Nutrition Protocol</t>
+          <t>PMS, cramps and appetite changes</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Hội Chứng Tiền Kinh Nguyệt (PMS), Đau Bụng Kinh &amp; Cơn Thèm Ăn Pha Hoàng Thể: Khoa Học Thần Kinh – Nội Tiết Và Phác Đồ Dinh Dưỡng</t>
+          <t>PMS, đau bụng kinh và thèm ăn: chăm sóc theo triệu chứng</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Đau bụng kinh, biến động cảm xúc, tích nước và cơn thèm đồ ngọt dữ dội trước kỳ kinh hoàn toàn không phải do 'tâm lý'—chúng được thúc đẩy bởi chất gây viêm Prostaglandin (PGF2α) tại tử cung, mức tăng trao đổi chất 100–250 kcal/ngày và sự sụt giảm Serotonin cuối pha Hoàng thể. Đây là phác đồ vi chất lâm sàng giúp làm dịu triệt để.</t>
+          <t>PMS có thể gồm thay đổi tâm trạng, khó ngủ, căng ngực và thèm ăn trước kỳ kinh.</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Hội chứng PMS và đau bụng kinh bắt nguồn từ ba cơ chế sinh hóa hoàn toàn có thể can thiệp: co thắt cơ trơn tử cung do Prostaglandin (PGF2α), sự sụt giảm chất dẫn truyền thần kinh Serotonin và GABA cuối pha Hoàng thể, cùng mức tăng chuyển hóa cơ bản (+100–250 kcal/ngày). Bổ sung Canxi (1.000–1.200 mg), Magie Glycinate (300–400 mg), Vitamin B6 (50–80 mg) và Omega-3 EPA/DHA trong pha Hoàng thể giúp giảm rõ rệt cơn đau và ổn định tâm trạng.</t>
+          <t>Ghi triệu chứng ít nhất hai chu kỳ, gồm thời điểm bắt đầu, lúc giảm và ảnh hưởng công việc. Duy trì bữa ăn cân bằng, vận động phù hợp và ngủ đủ; dùng nhật ký để trao đổi về lựa chọn điều trị nếu cần.</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>HO-06 (Symptom logs: severe mood swings, depression, anxiety), REC-03 (Chronic low recovery in late luteal)</t>
+          <t>PMS, cramps and appetite changes (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>Hantsoo &amp; Epperson (Curr Psychiatry Rep, 2015); Yonkers et al. (Lancet, 2008); DSM-5 PMDD Criteria</t>
+          <t>https://www.nhs.uk/conditions/pre-menstrual-syndrome/</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1905,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Understanding Female Libido</t>
+          <t>Understanding sexual desire in women</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -1888,7 +1915,7 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_09)</t>
+          <t>Revised — WH_09; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1898,32 +1925,32 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>The Science of Female Libido: Hormonal Drivers, Autonomic Balance &amp; Desire</t>
+          <t>Understanding sexual desire in women</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>Giải Mã Ham Muốn Nữ Giới: Động Lực Hormone, Trương Lực Thần Kinh &amp; Cơ Chế Hưng Phấn Đa Tầng</t>
+          <t>Ham muốn nữ giới: nhiều yếu tố cùng góp phần</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>Khác với nam giới vốn có cơ chế ham muốn mang tính bộc phát và phụ thuộc chủ yếu vào testosterone, ham muốn ở phụ nữ là một hệ thống phản ứng sinh học đa tầng phức tạp. Khám phá Mô hình Kiểm soát Kép (Dual Control Model), vai trò của oxytocin và lý do vì sao chỉ số HRV cao trên đồng hồ là điều kiện tiên quyết cho sự thăng hoa phòng the.</t>
+          <t>Ham muốn có thể thay đổi do sức khỏe, thuốc, stress, mối quan hệ, đau hoặc thay đổi giai đoạn sống.</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Hưng phấn ở phụ nữ vận hành theo cơ chế 'nhả chân phanh' (hạ cortisol, tăng HRV phó giao cảm) trước khi có thể 'nhấn chân ga' (kích hoạt dopamine và oxytocin). Bất kỳ tình trạng căng thẳng mãn tính hay kiệt sức nào cũng sẽ tự động kích hoạt hệ thống ức chế tình dục (SIS) của não bộ.</t>
+          <t>Nếu thay đổi gây khó chịu, ghi thời điểm bắt đầu, thuốc và các triệu chứng như khô hoặc đau. Trao đổi với bạn tình về sự thoải mái và mong muốn; có thể tìm tư vấn để xác định phần cần hỗ trợ.</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>REC-01 (HRV as indicator of parasympathetic safety), SL-11 (Sleep need satisfaction drives sexual vitality)</t>
+          <t>Understanding sexual desire in women (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>Basson (Obstet Gynecol, 2001 - Dual Control Model); Cappelletti &amp; Wallen (Horm Behav, 2016); Bancroft (2009)</t>
+          <t>https://www.nhs.uk/symptoms/loss-of-libido/</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1965,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Why Sexual Desire Changes Throughout Your Cycle</t>
+          <t>Cycle-related mood changes without fixed peaks</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -1948,7 +1975,7 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_10)</t>
+          <t>Revised — WH_10; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1958,32 +1985,32 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>The Desire Curve: Tracking Libido Peaks from Follicular Surge to Luteal Dip</t>
+          <t>Cycle-related mood changes without fixed peaks</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Đường Cong Cảm Xúc: Vì Sao Hưng Phấn Đạt Đỉnh Khi Rụng Trứng &amp; Hạ Nhiệt Cuối Kỳ?</t>
+          <t>Cảm xúc theo chu kỳ: không phải ai cũng có đỉnh hưng phấn lúc rụng trứng</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Nghiên cứu sinh hóa hormone của Roney &amp; Simmons (2013) khẳng định ham muốn tình dục ở nữ giới dao động có quy luật toán học theo từng ngày của chu kỳ kinh nguyệt. Khám phá lý do tại sao tự nhiên lại lập trình đỉnh hưng phấn vào cửa sổ thụ thai, và cách progesterone đưa cơ thể về trạng thái bảo tồn năng lượng trong pha hoàng thể.</t>
+          <t>PMS có thể gây khó chịu hoặc thay đổi tâm trạng trước kỳ kinh ở một số người.</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>Đỉnh ham muốn tự nhiên của bạn xuất hiện vào các ngày 11–15 của chu kỳ (khi estrogen và testosterone chạm đỉnh), trong khi sự suy giảm ham muốn ở pha hoàng thể là phản ứng sinh tồn để nuôi dưỡng tổ ấm. Hãy đồng bộ hóa đời sống lứa đôi theo nhịp sinh học này để giải phóng bản thân khỏi áp lực.</t>
+          <t>Ghi cảm xúc, giấc ngủ và sự kiện đáng chú ý ít nhất hai chu kỳ. Chọn một thay đổi thực tế như giờ nghỉ đều hoặc giảm lịch quá tải khi khó chịu. Chia sẻ nhật ký nếu cần tư vấn.</t>
         </is>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>HO-04 (Ovulatory phase window), HO-05 (Cycle progress tracking), appleSleepingWristTemperature</t>
+          <t>Cycle-related mood changes without fixed peaks (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
-          <t>Roney &amp; Simmons (Horm Behav, 2013); Bullivant et al. (Arch Sex Behav, 2004); Gangestad et al. (2007)</t>
+          <t>https://www.nhs.uk/conditions/pre-menstrual-syndrome/</t>
         </is>
       </c>
     </row>
@@ -1998,7 +2025,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Vaginal Health: What's Normal and What's Not?</t>
+          <t>Vaginal discharge and pH: useful signs and limits</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -2008,7 +2035,7 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_11)</t>
+          <t>Revised — WH_11; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -2018,32 +2045,32 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>The Vaginal Microbiome &amp; pH: Decoding Flora Balance, Odor &amp; Discharge</t>
+          <t>Vaginal discharge and pH: useful signs and limits</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Hệ Vi Sinh Âm Đạo &amp; Độ pH: Cách Đọc Vị Sức Khỏe Vùng Kín Chuẩn Y Khoa</t>
+          <t>Dịch tiết âm đạo và pH: dấu hiệu nào đáng chú ý?</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>Âm đạo là một hệ sinh thái tự làm sạch tinh vi được bảo vệ bởi hàng tỷ vi khuẩn Lactobacillus. Hiểu rõ sự tương tác giữa estrogen, glycogen và độ pH từ 3.8 đến 4.5 giúp bạn dễ dàng phân biệt dịch tiết sinh lý bình thường theo chu kỳ với các dấu hiệu cảnh báo viêm nhiễm cần can thiệp y khoa.</t>
+          <t>Dịch tiết có thể thay đổi bình thường theo chu kỳ.</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>Khí hư thay đổi từ lỏng trong suốt sang đục dính là hoàn toàn sinh lý theo dao động estrogen. Hãy bảo tồn lớp vi sinh vật tự nhiên bằng cách kiêng tuyệt đối thụt rửa sâu, chọn quần lót cotton thoáng khí và theo dõi triệu chứng mùi hôi hoặc ngứa rát song hành cùng pha chu kỳ trên ứng dụng.</t>
+          <t>Vệ sinh phần ngoài nhẹ nhàng, tránh thụt rửa và sản phẩm gây kích ứng. Khi có triệu chứng mới, ghi thời điểm và sản phẩm gần đây đã dùng; ưu tiên khám thay vì tự chọn kháng sinh hoặc thuốc nấm.</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>HO-06 (Vaginal discharge logging: normal, clot-like, odor), HealthKit vaginalDischargeCategory</t>
+          <t>Vaginal discharge and pH: useful signs and limits (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr">
         <is>
-          <t>Ravel et al. (PNAS, 2011 - Vaginal Community State Types); Witkin &amp; Linhares (BJOG, 2017); ACOG Guidelines</t>
+          <t>https://www.acog.org/womens-health/faqs/vulvovaginal-health</t>
         </is>
       </c>
     </row>
@@ -2058,7 +2085,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Pain During Sex: Common Causes &amp; When to Seek Help</t>
+          <t>Pain during sex: finding the cause</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -2068,7 +2095,7 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_12)</t>
+          <t>Revised — WH_12; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -2078,32 +2105,32 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Unpacking Dyspareunia: Musculoskeletal, Hormonal &amp; Structural Triggers</t>
+          <t>Pain during sex: finding the cause</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Đau Rát Khi Quan Hệ (Dyspareunia): Căn Nguyên Cơ Học, Nội Tiết &amp; Giải Pháp Điều Trị</t>
+          <t>Đau khi quan hệ: không cần cố chịu đựng</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>Đau rát khi quan hệ tình dục không bao giờ là điều bạn phải cắn răng chịu đựng hay xem là chuyện 'bình thường'. Từ sự co thắt quá mức của các bó cơ sàn chậu đến tình trạng suy giảm estrogen hay lạc nội mạc tử cung, y học hiện đại có các phác đồ chuẩn xác để chữa lành tận gốc chứng giao hợp đau (Dyspareunia).</t>
+          <t>Đau có thể liên quan khô, kích ứng, nhiễm trùng, sàn chậu hoặc bệnh vùng chậu.</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>Nếu bạn bị đau rát khi quan hệ, giải pháp đầu tiên không phải là 'cố gắng chịu đựng' hay tập Kegel siết chặt cơ. Hãy phân biệt đau nông tại cửa mình (cần khám nơ-ron tiền đình, phục hồi màng nhầy) hay đau sâu trong ổ bụng (cần tầm soát lạc nội mạc, nang buồng trứng), đồng thời ưu tiên các bài tập hạ trương lực cơ sàn chậu.</t>
+          <t>Dừng hoạt động gây đau và trao đổi rõ với bạn tình. Có thể thử chất bôi trơn phù hợp và hoạt động không đau nếu cả hai muốn. Ghi đau nông hay sâu, thời điểm và dấu hiệu đi kèm để trao đổi khi khám.</t>
         </is>
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>HO-06 (Pelvic pain self-report), STR-01 (Autonomic tension &amp; high stress driving pelvic floor guarding)</t>
+          <t>Pain during sex: finding the cause (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>Seehusen et al. (Am Fam Physician, 2014); Bergeron et al. (J Sex Med, 2011); ACOG Practice Bulletin #226</t>
+          <t>https://www.acog.org/womens-health/faqs/when-sex-is-painful</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2145,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Pelvic Floor Health: Why It Matters</t>
+          <t>Pelvic-floor function in women</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -2128,7 +2155,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_13)</t>
+          <t>Revised — WH_13; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -2138,32 +2165,32 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>The Female Pelvic Floor Engine: Continence, Core Stability &amp; Sexual Vitality</t>
+          <t>Pelvic-floor function in women</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Sàn Chậu Nữ Giới: Chiếc Võng Cơ Học Quyết Định Độ Vững Vàng Vùng Lõi &amp; Bản Lĩnh Phòng The</t>
+          <t>Sàn chậu nữ: sức mạnh cần đi cùng khả năng thả lỏng</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>Sàn chậu không chỉ liên quan đến câu chuyện tiểu són hay sinh nở—đây là nền tảng cơ học nâng đỡ toàn bộ nội tạng, tạo lực bộc phát trong từng bước chạy và điều phối cực khoái trong đời sống lứa đôi. Khám phá cách vận hành 'chiếc hộp áp lực ổ bụng' và lý do tại sao tập siết cơ không đúng cách có thể phản tác dụng.</t>
+          <t>Sàn chậu góp phần nâng đỡ cơ quan và kiểm soát tiểu tiện.</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>Sàn chậu khỏe mạnh không phải là sàn chậu luôn siết chặt, mà là sàn chậu có khả năng co giãn linh hoạt theo từng nhịp thở. Hãy kết hợp thở cơ hoành (Piston Breathing) trong từng rep tập kháng lực và lắng nghe các tín hiệu rò rỉ tiểu hoặc tức nặng vùng chậu trên ứng dụng để điều chỉnh áp lực kịp thời.</t>
+          <t>Nếu có rò tiểu, nặng vùng chậu hoặc không chắc kỹ thuật, gặp chuyên viên để kiểm tra khả năng co và thả. Trong khi tập, thở tự nhiên, tránh siết bụng và cho cơ nghỉ đầy đủ.</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
         <is>
-          <t>STR-01 (Core intra-abdominal strain), ACT-01 (Pelvic stability during running/jumping impacts)</t>
+          <t>Pelvic-floor function in women (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>Bø et al. (Int Urogynecol J, 2017); Dumoulin et al. (Cochrane Database Syst Rev, 2018); Kegel (1948)</t>
+          <t>https://www.nhs.uk/conditions/urinary-incontinence/treatment/</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2205,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>How Your Menstrual Cycle May Affect Exercise</t>
+          <t>Cycle-aware training without rigid phase rules</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -2188,7 +2215,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Completed (Mapped to DM_WH_01)</t>
+          <t>Revised — DM_WH_01; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -2198,32 +2225,32 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Cycle-Synced Training: How to Periodize Strength, HIIT, and Recovery Across Your Menstrual Cycle</t>
+          <t>Cycle-aware training without rigid phase rules</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Tập Luyện Đồng Bộ Chu Kỳ (Cycle-Synced Training): Cách Phân Kỳ Sức Mạnh, HIIT Và Phục Hồi Theo Nội Tiết Tố</t>
+          <t>Tập theo chu kỳ: ưu tiên triệu chứng hơn lịch pha cố định</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Vì sao cùng một giáo án nâng tạ hay chạy bộ lại mang đến cảm giác nhẹ nhàng ở Tuần 2 nhưng lại vắt kiệt sức lực ở Tuần 4 của chu kỳ? Khám phá khoa học nội tiết thể thao từ Tiến sĩ Stacy Sims và WHOOP Menstrual Cycle Coaching để tối ưu hóa tải tập luyện theo nhịp điệu Estrogen và Progesterone.</t>
+          <t>Tổng quan hệ thống cho thấy ảnh hưởng trung bình của pha chu kỳ lên hiệu suất thường nhỏ và bằng chứng còn hạn chế.</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Hãy dồn các buổi tập tạ nặng, cường độ cao ngắt quãng (HIIT) và mục tiêu phá kỷ lục cá nhân vào giai đoạn Nang trứng và Rụng trứng (Ngày 3–15) khi Estrogen tối ưu hóa tổng hợp protein cơ bắp và sử dụng glycogen. Sang nửa cuối pha Hoàng thể (Ngày 20–28), hãy chuyển sang Cardio Zone 2 bền bỉ, rèn kỹ thuật, tăng lượng đạm (1.8–2.2 g/kg) và chủ động làm mát cơ thể.</t>
+          <t>Giữ kế hoạch tập có thể duy trì, ghi thêm đau, năng lượng và cảm giác gắng sức. Nếu nhận thấy mẫu triệu chứng lặp lại qua vài chu kỳ, linh hoạt đổi buổi hoặc giảm tải theo nhu cầu thực tế.</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>HO-04 (Phase estimation), STR-01 (Daily Strain targets matching cycle phases: 14-18 in Follicular, 8-12 in Luteal)</t>
+          <t>Cycle-aware training without rigid phase rules (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>Sims et al. (PLOS ONE / BMJ, 2021); McNulty et al. (Sports Med, 2020); WHOOP The Locker Menstrual Coaching</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/32661839/</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2265,7 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Training During Your Period: What You Should Know</t>
+          <t>Exercising during your period</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -2248,7 +2275,7 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_15)</t>
+          <t>Revised — WH_15; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -2258,32 +2285,32 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Exercising on Your Period: Biomechanics, Uterine Blood Flow &amp; Deload Strategy</t>
+          <t>Exercising during your period</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>Tập Gì Khi Đang Có Kinh? Lưu Lượng Máu Tử Cung &amp; Chiến Lược Tập Luyện Phục Hồi</t>
+          <t>Tập khi có kinh: chọn cường độ theo mức dễ chịu</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>Nhiều phụ nữ phân vân liệu có nên tập luyện khi đang có kinh hay nên nằm yên nghỉ ngơi hoàn toàn. Khoa học thể thao chứng minh vận động cường độ nhẹ đến vừa kích hoạt giải phóng Endorphin giảm đau tự nhiên và tăng cường lưu thông máu vùng chậu. Khám phá cách điều chỉnh tải trọng (Deload) chuẩn xác theo tín hiệu thiết bị đeo.</t>
+          <t>Có kinh không tự tạo chống chỉ định vận động.</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>Bạn không cần ngừng tập khi có kinh, nhưng hãy hạ cường độ từ ngưỡng bộc phát (RPE 8–10) xuống mức kích thích phục hồi (RPE 5–6) trong 48 giờ đầu. Ưu tiên đi bộ nhanh, yoga giãn mạc hoặc bơi nhẹ để hạ nồng độ prostaglandin gây co thắt tử cung.</t>
+          <t>Thử buổi tập ngắn hơn hoặc cường độ dễ chịu khi có triệu chứng; giữ kế hoạch bình thường nếu cảm thấy khỏe. Theo dõi đau và lượng chảy máu, chuẩn bị sản phẩm kinh nguyệt phù hợp và ăn uống đủ.</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr">
         <is>
-          <t>HO-01 (Period flow tracking), REC-02 (RHR drop and HRV rebound on Days 2-4 signaling physiological relief)</t>
+          <t>Exercising during your period (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L19" s="7" t="inlineStr">
         <is>
-          <t>Dehnavi et al. (J Educ Health Promot, 2018); Armour et al. (BMC Complement Altern Med, 2019)</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/32661839/</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2325,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Understanding Recovery &amp; HRV in Women</t>
+          <t>HRV changes across the menstrual cycle</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -2308,7 +2335,7 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_16)</t>
+          <t>Revised — WH_16; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -2318,32 +2345,32 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Female HRV Biometrics: Why Your Parasympathetic Baseline Shifts Across the Month</t>
+          <t>HRV changes across the menstrual cycle</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>Biến Thiên Nhịp Tim (HRV) Ở Nữ Giới: Giải Mã Bước Giảm Tự Nhiên Sau Khi Rụng Trứng</t>
+          <t>HRV thay đổi theo chu kỳ: so với nền riêng của bạn</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>Nếu bạn nhận thấy điểm Biến thiên nhịp tim (HRV) của mình đột ngột sụt giảm 10–15% và điểm Phục hồi chuyển sang màu vàng trong hai tuần cuối của tháng, đừng hoảng sợ rằng bạn bị kiệt sức. Đó là một hiện tượng sinh lý học bình thường do progesterone chi phối hệ thần kinh thực vật.</t>
+          <t>Tổng quan nghiên cứu ghi nhận hoạt động phế vị có thể thay đổi theo pha chu kỳ ở cấp độ nhóm.</t>
         </is>
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>Đừng so sánh chỉ số HRV pha hoàng thể với pha nang trứng. Hãy xây dựng hai đường cơ sở (Baseline) riêng biệt cho cơ thể: một mức nền cao ở nửa đầu chu kỳ (nhờ estrogen kích hoạt hệ phó giao cảm) và một mức nền thấp hơn ở nửa sau chu kỳ (do progesterone kích hoạt hệ giao cảm và tăng nhiệt độ cơ thể).</t>
+          <t>Đọc HRV cùng ngày kinh, giấc ngủ, bệnh gần đây và tải tập. So với nền trên cùng thiết bị trong nhiều chu kỳ nếu việc ghi nhận không gây áp lực. Điều chỉnh theo triệu chứng thay vì cố nâng điểm.</t>
         </is>
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>REC-01 (HRV RMSSD baseline), REC-03 (Female recovery score compensation), Apple heartRateVariabilitySDNN</t>
+          <t>HRV changes across the menstrual cycle (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
-          <t>Schmalenberger et al. (Psychoneuroendocrinology, 2019); Sims et al. (2021); WHOOP Science</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/31726666/</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2385,7 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Strength Training Benefits for Women's Health</t>
+          <t>Strength training for women</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -2368,7 +2395,7 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_17)</t>
+          <t>Revised — WH_17; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -2378,32 +2405,32 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Resistance Training for Women: Bone Mineral Density, Insulin Sensitivity &amp; Longevity</t>
+          <t>Strength training for women</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>Tập Kháng Lực Cho Phái Đẹp: Mật Độ Xương, Độ Nhạy Insulin &amp; Trẻ Hóa Chuyển Hóa</t>
+          <t>Tập sức mạnh cho nữ: xây thói quen lâu dài</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>Tập tạ không khiến phụ nữ bị 'đô con' hay thô kệch—đó là tấm khiên y khoa vững chắc nhất để bảo vệ mật độ xương trước nguy cơ loãng xương, tối ưu hóa độ nhạy insulin và duy trì tốc độ chuyển hóa cơ bản suốt cuộc đời. Khám phá khoa học đằng sau các bài tập tạ nặng và thử nghiệm lâm sàng LIFTMOR.</t>
+          <t>Tập sức mạnh là một phần của vận động lành mạnh ở người trưởng thành.</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>Phụ nữ đạt đỉnh mật độ xương ở tuổi 25–30 và mất xương nhanh chóng sau mãn kinh. Các bài tập cardio nhẹ không đủ lực kích hoạt tế bào tạo xương; bạn cần các bài tập kháng lực đa khớp (Squat, Deadlift, Overhead Press) với mức tạ từ 70–85% 1RM ít nhất 2–3 lần mỗi tuần.</t>
+          <t>Chọn bài phù hợp kinh nghiệm, học kỹ thuật và để cơ thể hồi phục giữa các buổi nặng. Người mới có thể bắt đầu nhẹ và tăng khi kiểm soát tốt. Kết hợp vận động tim mạch và ăn đủ năng lượng.</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
-          <t>ACT-01 (Muscular Load / Strain), HS-01 (Biological Age reduction via skeletal muscle preservation)</t>
+          <t>Strength training for women (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>Watson et al. (J Bone Miner Res, 2018 - LIFTMOR Trial); Westcott (Curr Sports Med Rep, 2012); ACOG</t>
+          <t>https://www.who.int/news-room/fact-sheets/detail/physical-activity</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2445,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Signs of Overtraining &amp; Low Energy Availability</t>
+          <t>REDs and low energy availability</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -2428,7 +2455,7 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_18)</t>
+          <t>Revised — WH_18; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -2438,32 +2465,32 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>RED-S &amp; Low Energy Availability: Recognizing Overtraining &amp; Hypothalamic Amenorrhea</t>
+          <t>REDs and low energy availability</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>Hội Chứng RED-S &amp; Thiếu Năng Lượng Sẵn Có: Hiểm Họa Mất Kinh &amp; Quá Tải Tập Luyện</t>
+          <t>REDs: khi ăn không đủ so với nhu cầu tập luyện</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>Mất kinh không phải là 'huy chương danh dự' chứng minh bạn tập luyện chăm chỉ hay giảm mỡ thành công; đó là hồi chuông báo động đỏ của cơ thể khi rơi vào Hội chứng Thiếu Hụt Năng Lượng Tương Đối Trong Thể Thao (RED-S). Tìm hiểu công thức tính năng lượng sẵn có và cách cứu vãn buồng trứng cùng khung xương trước khi quá muộn.</t>
+          <t>Thiếu năng lượng sẵn có kéo dài có thể ảnh hưởng nhiều hệ cơ thể, gồm xương, sinh sản và hiệu suất.</t>
         </is>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>Nếu chu kỳ kinh nguyệt của bạn bị trễ trên 35 ngày hoặc biến mất hoàn toàn kết hợp với tập luyện nặng và ăn kiêng gắt gao, bạn đang bị thiếu năng lượng sẵn có (&lt; 30 kcal/kg FFM/ngày). Hãy ngừng ngay việc cắt giảm tinh bột, giảm bớt tải trọng tập luyện (Strain) và theo dõi sự phục hồi của thân nhiệt cùng HRV trên ứng dụng.</t>
+          <t>Nếu mệt, hồi phục kém hoặc chu kỳ thay đổi cùng tải tập cao, xem lại lượng ăn và lịch tập với bác sĩ hoặc chuyên gia dinh dưỡng thể thao. Ghi xu hướng triệu chứng; không chờ cân nặng xuống thấp mới tìm hỗ trợ.</t>
         </is>
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>HO-02 (Cycle tracking: alert when cycle &gt;35d or missed), REC-01 (Depressed HRV), STR-01 (Chronic overstraining)</t>
+          <t>REDs and low energy availability (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L22" s="7" t="inlineStr">
         <is>
-          <t>Mountjoy et al. (Br J Sports Med, IOC Consensus 2018/2023); De Souza et al. (Hum Reprod Update, 2014)</t>
+          <t>https://bjsm.bmj.com/content/57/17/1073</t>
         </is>
       </c>
     </row>
@@ -2478,7 +2505,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Why Sleep May Change Before Your Period</t>
+          <t>Sleep difficulties before your period</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
@@ -2488,7 +2515,7 @@
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_19)</t>
+          <t>Revised — WH_19; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -2498,32 +2525,32 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>The Luteal Insomnia Effect: How Progesterone &amp; Thermoregulation Fragment Sleep</t>
+          <t>Sleep difficulties before your period</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>Hội Chứng Khó Ngủ Tiền Kinh Nguyệt: Vì Sao Thân Nhiệt Tăng Làm Gián Đoạn Giấc Ngủ REM?</t>
+          <t>Khó ngủ trước kỳ kinh: chăm sóc triệu chứng, không chạy theo REM</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>Nếu bạn thường xuyên trằn trọc, đổ mồ hôi đêm hoặc tỉnh giấc giữa chừng vào tuần lễ trước kỳ kinh, đó không phải là sự trùng hợp ngẫu nhiên. Sự gia tăng nồng độ progesterone đẩy thân nhiệt cơ bản lên cao, làm xáo trộn cơ chế làm mát tự nhiên của não bộ và cắt vụn các chu kỳ ngủ sâu.</t>
+          <t>Khó ngủ có thể là một phần của PMS, đồng thời đau, môi trường và stress cũng ảnh hưởng.</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>Để đi vào giấc ngủ sâu, nhiệt độ cơ thể cần hạ xuống khoảng 1°C. Ở pha hoàng thể, progesterone ngăn chặn bước hạ nhiệt này. Hãy chủ động làm mát cơ thể: hạ điều hòa phòng ngủ xuống 18°C–19°C, tắm nước ấm trước khi ngủ 90 phút để kích thích giãn mạch ngoại vi, và hạn chế ăn khuya.</t>
+          <t>Ghi lịch ngủ và triệu chứng qua ít nhất hai chu kỳ. Giữ giờ ngủ tương đối đều, phòng thoải mái và xử trí đau theo tư vấn phù hợp. Nếu app làm bạn lo hơn, thử ưu tiên mức tỉnh táo thay cho tỷ lệ giai đoạn ngủ.</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
-          <t>SL-01 (Sleep performance dip in luteal), SL-11 (Increased sleep need), appleSleepingWristTemperature</t>
+          <t>Sleep difficulties before your period (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
-          <t>Baker &amp; Driver (Sleep Med Rev, 2007); Shechter &amp; Boivin (Sleep Med Clin, 2018); Oura Ring Sleep Data</t>
+          <t>https://www.nhs.uk/conditions/pre-menstrual-syndrome/</t>
         </is>
       </c>
     </row>
@@ -2538,7 +2565,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>How Stress Can Affect Your Menstrual Cycle</t>
+          <t>Stress and a late period: considering other causes</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
@@ -2548,7 +2575,7 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_20)</t>
+          <t>Revised — WH_20; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -2558,32 +2585,32 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Cortisol vs. The Ovaries: How Chronic Stress Shuts Down Ovulation</t>
+          <t>Stress and a late period: considering other causes</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>Khi Cortisol Áp Đảo Buồng Trứng: Cơ Chế Căng Thẳng Làm Trễ Kinh &amp; Ức Chế Rụng Trứng</t>
+          <t>Stress và trễ kinh: cần xem xét những nguyên nhân nào?</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>Một kỳ thi căng thẳng, một dự án áp lực cao hoặc cú sốc tinh thần có thể khiến kỳ kinh của bạn biến mất cả tháng. Đó không phải là lỗi của buồng trứng, mà là cơ chế sinh tồn ưu việt của não bộ: khi trục HPA phát tín hiệu nguy hiểm, vùng hạ đồi sẽ lập tức hoãn việc rụng trứng để bảo vệ bạn khỏi việc mang thai trong hoàn cảnh ngặt nghèo.</t>
+          <t>Stress có thể liên quan thay đổi chu kỳ, nhưng mang thai, thay đổi cân nặng, vận động nhiều, thuốc và bệnh lý cũng có thể làm trễ kinh.</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>Khi gặp căng thẳng nặng, trứng không thể rụng đúng hạn khiến chu kỳ bị kéo dài. Đừng uống thuốc ép kinh bừa bãi. Hãy theo dõi điểm Căng thẳng Thần kinh (Stress Monitor) và HRV trên thiết bị đeo; khi nhịp tim nghỉ ngơi hạ nhiệt và hệ phó giao cảm hồi phục, buồng trứng sẽ tự động kích hoạt rụng trứng trở lại.</t>
+          <t>Nếu có khả năng mang thai, thử thai đúng thời điểm. Ghi lại thay đổi lịch sống, khẩu phần và tải tập; ưu tiên ngủ, ăn đều và cách giảm áp lực khả thi. Theo dõi nếu kỳ kinh vẫn chưa trở lại.</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>HO-03 (Next-period delayed alert), REC-03 (High stress score days), REC-01 (Autonomic imbalance)</t>
+          <t>Stress and a late period: considering other causes (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L24" s="7" t="inlineStr">
         <is>
-          <t>Berga &amp; Loucks (Fertil Steril); Schliep et al. (Am J Epidemiol, 2015); Chrousos et al. (Ann N Y Acad Sci)</t>
+          <t>https://www.nhs.uk/symptoms/missed-or-late-periods/</t>
         </is>
       </c>
     </row>
@@ -2598,7 +2625,7 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Nutrition Essentials for Women's Health</t>
+          <t>Nutrition across the cycle</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
@@ -2608,7 +2635,7 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_21)</t>
+          <t>Revised — WH_21; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -2618,32 +2645,32 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Fueling the Female Metabolism: Macronutrient Timing Across Follicular &amp; Luteal Phases</t>
+          <t>Nutrition across the cycle</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>Dinh Dưỡng Đồng Bộ Nội Tiết: Chiến Lược Bổ Sung Tinh Bột, Protein &amp; Chất Béo Thông Minh</t>
+          <t>Dinh dưỡng quanh chu kỳ: đủ năng lượng trước khi theo thực đơn theo pha</t>
         </is>
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>Cơ thể phụ nữ không phải là một cỗ máy chuyển hóa bất biến như nam giới; khả năng đốt mỡ, dung nạp tinh bột và phân hủy protein thay đổi rõ rệt qua từng tuần theo nồng độ hormone. Áp dụng dinh dưỡng đồng bộ chu kỳ (Cycle-Synced Nutrition) giúp bạn đập tan cơn thèm đồ ngọt tiền kinh nguyệt và tối ưu hiệu suất thể thao.</t>
+          <t>Ăn đủ và đa dạng quan trọng hơn một thực đơn cứng theo ngày chu kỳ.</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>Tận dụng độ nhạy insulin cao ở nửa đầu chu kỳ (Pha Nang trứng) để nạp tinh bột phức hợp phục vụ các bài tập nặng. Ở nửa sau chu kỳ (Pha Hoàng thể), khi tốc độ chuyển hóa cơ bản tăng 100–250 kcal/ngày nhưng cơ thể dễ bị dị hóa cơ bắp, hãy tăng lượng protein lên 1.8–2.0g/kg và bổ sung chất béo lành mạnh.</t>
+          <t>Duy trì bữa chính có nguồn đạm, tinh bột, rau và chất béo phù hợp; thêm bữa phụ khi đói hoặc tập nhiều. Nếu ăn kiêng làm mệt, mất kinh hay giảm hiệu suất, xem lại tổng năng lượng với người có chuyên môn.</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
-          <t>STR-01 (Caloric &amp; metabolic expenditure variation), HS-01 (Nutritional metabolic efficiency)</t>
+          <t>Nutrition across the cycle (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>Oosthuyse &amp; Bosch (Sports Med, 2010); Campbell et al. (J Int Soc Sports Nutr, 2018); Sims (ROAR, 2016)</t>
+          <t>https://www.who.int/news-room/fact-sheets/detail/healthy-diet</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2685,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Iron Deficiency &amp; Heavy Periods</t>
+          <t>Heavy periods and iron deficiency</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -2668,7 +2695,7 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_22)</t>
+          <t>Revised — WH_22; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -2678,32 +2705,32 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Menorrhagia &amp; Ferritin: Overcoming Hidden Iron Deficiency &amp; Fatigue</t>
+          <t>Heavy periods and iron deficiency</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>Kinh Nguyệt Ra Nhiều &amp; Thiếu Máu: Dấu Hiệu Tụt Ferritin &amp; Phác Đồ Bù Sắt Khoa Học</t>
+          <t>Kinh nhiều và thiếu sắt: xét nghiệm trước khi tự bổ sung</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>Bạn cảm thấy tim đập thình thịch khi leo cầu thang, hụt hơi khi chạy bộ dù kết quả xét nghiệm máu cho thấy nồng độ Hemoglobin 'bình thường'? Rất có thể bạn đang bị thiếu sắt tiềm ẩn (Tụt Ferritin) do kinh nguyệt ra nhiều (Menorrhagia). Khám phá cách chẩn đoán và phác đồ bù sắt chuẩn y học thể thao.</t>
+          <t>Kinh nhiều có thể dẫn đến thiếu sắt hoặc thiếu máu.</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>Đừng chỉ kiểm tra nồng độ Hemoglobin; hãy yêu cầu bác sĩ xét nghiệm Ferritin huyết thanh (mục tiêu tối ưu cho phụ nữ vận động là &gt; 50 ng/mL). Nếu bạn phải thay băng vệ sinh sau mỗi 1–2 giờ hoặc có cục máu đông lớn hơn đồng xu, hãy bổ sung sắt hữu cơ dạng Sắt Bisglycinate uống cách ngày kết hợp cùng Vitamin C.</t>
+          <t>Ghi số ngày chảy máu, tần suất thay sản phẩm và ảnh hưởng sinh hoạt. Hỏi bác sĩ về xét nghiệm máu và nguyên nhân chảy máu; nếu được kê sắt, theo hướng dẫn và lịch kiểm tra lại.</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>HO-01 (Menstrual flow intensity: heavy), REC-02 (Elevated RHR from compensatory cardiac output), VO2 Max dip</t>
+          <t>Heavy periods and iron deficiency (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L26" s="7" t="inlineStr">
         <is>
-          <t>Fraser et al. (Int J Gynaecol Obstet, 2015); Peeling et al. (Eur J Appl Physiol, 2008); WHO Iron Guidelines</t>
+          <t>https://www.nhs.uk/conditions/heavy-periods/</t>
         </is>
       </c>
     </row>
@@ -2718,7 +2745,7 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Understanding Fertility &amp; Conception</t>
+          <t>Timing intercourse when trying to conceive</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
@@ -2728,7 +2755,7 @@
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_23)</t>
+          <t>Revised — WH_23; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -2738,32 +2765,32 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>The Conception Timeline: Gamete Lifespans, Capacitation &amp; The 6-Day Window</t>
+          <t>Timing intercourse when trying to conceive</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>Dòng Thời Gian Thụ Thai: Tuổi Thọ Giao Tử &amp; Nghệ Thuật Canh Cửa Sổ Thụ Thai Chuẩn Xác</t>
+          <t>Canh thời điểm thụ thai: giảm áp lực phải đúng một ngày</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>Nhiều cặp đôi lầm tưởng rằng chỉ có thể thụ thai vào đúng ngày rụng trứng, dẫn đến việc bỏ lỡ những thời điểm vàng quý giá nhất. Khám phá bí mật tuổi thọ giao tử, hiện tượng biến đổi tinh trùng (Capacitation) và cách công nghệ thiết bị đeo giúp bạn xác định chuẩn xác cửa sổ sinh sản 6 ngày.</t>
+          <t>Khả năng thụ thai cao hơn quanh các ngày trước rụng trứng, nhưng thời điểm thực tế khó biết chính xác bằng lịch.</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>Trứng chỉ sống được 12–24 giờ sau khi rụng, nhưng tinh trùng có thể sống khỏe mạnh tới 3–5 ngày trong dịch nhầy cổ tử cung giàu estrogen. Để tối đa hóa cơ hội có thai, hãy quan hệ vào 1–2 ngày TRƯỚC KHI rụng trứng thay vì chờ đến khi nhiệt độ cơ thể đã tăng vọt.</t>
+          <t>ASRM gợi ý quan hệ mỗi một đến hai ngày trong giai đoạn dễ thụ thai nếu phù hợp với cả hai. Nếu việc theo dõi gây căng thẳng, có thể ưu tiên nhịp quan hệ đều thay vì liên tục kiểm tra dữ liệu.</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>HO-04 (Predictive ovulation window), appleSleepingWristTemperature biphasic shift (Wang 2025)</t>
+          <t>Timing intercourse when trying to conceive (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
-          <t>Wilcox et al. (Hum Reprod, 1998); Stanford et al. (Obstet Gynecol, 2002); American Society for Reproductive Medicine</t>
+          <t>https://integration.asrm.org/globalassets/_asrm/practice-guidance/practice-guidelines/pdf/optimizing_natural_fertility.pdf</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2805,7 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Early Signs of Pregnancy</t>
+          <t>Early pregnancy signs and reliable testing</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -2788,7 +2815,7 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_24)</t>
+          <t>Revised — WH_24; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -2798,32 +2825,32 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Implantation Biometrics: Early hCG Triggers, Wearable Temperature &amp; Subtle Clues</t>
+          <t>Early pregnancy signs and reliable testing</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>Dấu Hiệu Thai Sớm: Sự Làm Tổ Của Phôi Nang, Đỉnh hCG &amp; Tín Hiệu Nhiệt Độ Thiết Bị Đeo</t>
+          <t>Dấu hiệu thai sớm: dùng que thử thay vì suy từ thiết bị đeo</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>Trước khi que thử thai xuất hiện 2 vạch rõ ràng, cơ thể bạn đã âm thầm diễn ra một cuộc cách mạng sinh học vi mô. Khi phôi nang làm tổ thành công vào nội mạc tử cung, các thuật toán trên thiết bị đeo thông minh có thể phát hiện bước nhảy thân nhiệt thứ ba (Triphasic BBT) và sự gia tăng nhịp tim nghỉ ngơi từ nhiều ngày trước kỳ kinh dự kiến.</t>
+          <t>Trễ kinh, căng ngực, mệt hoặc buồn nôn có thể xuất hiện khi mang thai nhưng cũng có nguyên nhân khác.</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>Dấu hiệu mang thai sớm nhất trên thiết bị đeo là biểu đồ nhiệt độ 3 pha (Triphasic pattern): nhiệt độ da ban đêm tiếp tục tăng bước nhảy thứ hai sau ngày 8–10 sau rụng trứng (DPO) thay vì hạ nhiệt chuẩn bị hành kinh, đi kèm nhịp tim nghỉ ngơi RHR tăng thêm 2–4 bpm và không có máu kinh xuất hiện.</t>
+          <t>Thử thai từ ngày đầu trễ kinh; nếu không biết ngày dự kiến, thử ít nhất 21 ngày sau lần quan hệ không bảo vệ gần nhất. Nếu âm tính quá sớm mà vẫn nghi có thai, thử lại theo hướng dẫn sau vài ngày.</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>HO-08 (Pregnancy insights: sustained high skin temp past day 18, rising RHR trend - Rowan 2022 BMC)</t>
+          <t>Early pregnancy signs and reliable testing (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L28" s="7" t="inlineStr">
         <is>
-          <t>Rowan et al. (BMC Pregnancy Childbirth, 2022); Cole (Reprod Biol Endocrinol, 2012); Wilcox et al. (NEJM, 1999)</t>
+          <t>https://www.nhs.uk/pregnancy/trying-for-a-baby/doing-a-pregnancy-test/</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2865,7 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>How Your Body Changes During Pregnancy</t>
+          <t>Body changes during pregnancy</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -2848,7 +2875,7 @@
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_25)</t>
+          <t>Revised — WH_25; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -2858,32 +2885,32 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Cardiovascular &amp; Metabolic Adaptations: What Happens During Each Trimester</t>
+          <t>Body changes during pregnancy</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>Chuyển Hóa Kỳ Diệu Khi Mang Thai: Cung Lượng Tim, Dung Tích Máu &amp; Biến Đổi Từng Tam Cá Nguyệt</t>
+          <t>Cơ thể thay đổi khi mang thai: theo dõi triệu chứng quan trọng</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>Mang thai tương đương với việc chạy một cuộc thi marathon kéo dài 40 tuần liên tục: thể tích máu tăng 50%, tim phải đập thêm 15.000 nhịp mỗi ngày và hệ thống mạch máu tái cấu trúc toàn diện. Tìm hiểu các biến đổi sinh học phi thường qua từng tam cá nguyệt từ công trình nghiên cứu thai kỳ liên tục của WHOOP.</t>
+          <t>Thai kỳ tạo nhiều thay đổi về tuần hoàn, tiêu hóa và cảm giác vận động.</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>Nhịp tim nghỉ ngơi tăng thêm 10–15 bpm và điểm HRV sụt giảm sâu trong thai kỳ là sự thích nghi tim mạch hoàn toàn bình thường để nuôi dưỡng thai nhi, không phải dấu hiệu kiệt sức. Nhịp tim đạt đỉnh quanh tuần thứ 30 và bắt đầu ổn định chuẩn bị cho cuộc chuyển dạ.</t>
+          <t>Duy trì lịch khám thai và hỏi đội ngũ chăm sóc về thay đổi bạn nhận thấy. Nếu dùng thiết bị đeo, xem dữ liệu như thông tin bổ sung và ghi triệu chứng đi kèm; không tự đặt mục tiêu giảm nhịp tim bằng hạn chế ăn hoặc tập quá sức.</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
         <is>
-          <t>HO-08 (Trimester RHR &amp; HRV trajectories - Rowan 2022 WHOOP pregnancy study; Adaimi 2025 Oura)</t>
+          <t>Body changes during pregnancy (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>Rowan et al. (2022); Sanghavi &amp; Rutherford (Circulation, 2014); Jasinski et al. (PLoS One, 2024)</t>
+          <t>https://www.nhs.uk/pregnancy/common-symptoms/common-health-problems/</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2925,7 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Safe Exercise During Pregnancy</t>
+          <t>Exercise during pregnancy</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -2908,7 +2935,7 @@
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_26)</t>
+          <t>Revised — WH_26; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -2918,32 +2945,32 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Prenatal Fitness Protocols: Safe Heart Rate Zones, Core Protection &amp; ACOG Guidelines</t>
+          <t>Exercise during pregnancy</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>Tập Luyện An Toàn Trong Thai Kỳ: Hướng Dẫn Y Khoa ACOG &amp; Các Vùng Nhịp Tim Tối Ưu</t>
+          <t>Vận động trong thai kỳ: trao đổi trước và theo dõi dấu hiệu dừng</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>Quan niệm cổ hủ cho rằng phụ nữ mang thai phải nằm yên dưỡng thai đã bị y học hiện đại bác bỏ hoàn toàn. Tập luyện đúng cách trong thai kỳ giúp giảm 50% nguy cơ tiểu đường thai kỳ, hạ tỷ lệ sinh mổ và bảo vệ vùng thắt lưng. Khám phá hướng dẫn an toàn chuẩn mực từ Đại học Sản Phụ khoa Hoa Kỳ (ACOG).</t>
+          <t>Nhiều người có thai kỳ không biến chứng có thể vận động và nhận lợi ích.</t>
         </is>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>Phụ nữ mang thai không có biến chứng nên duy trì ít nhất 150 phút vận động cường độ vừa phải mỗi tuần. Sử dụng 'Bài kiểm tra nói chuyện' (Talk Test) hoặc giữ nhịp tim dưới 60%–70% nhịp tim tối đa; tránh tuyệt đối các bài tập nằm ngửa sau tuần 16, các môn thể thao va chạm mạnh và các môi trường quá nóng.</t>
+          <t>Trao đổi trong khám thai về hoạt động đang làm và các điều chỉnh cần thiết. Nếu mới bắt đầu, tăng dần; dùng cảm giác gắng sức và khả năng trò chuyện thay vì ép đạt nhịp tim cụ thể. Tránh quá nóng và hoạt động có nguy cơ va chạm hoặc ngã.</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>ACT-01 (Safe prenatal strain monitoring), STR-01 (Preventing heat stress &amp; extreme heart rate peaks)</t>
+          <t>Exercise during pregnancy (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>ACOG Committee Opinion No. 804 (2020); Mottola et al. (Br J Sports Med, Canadian Guidelines 2019)</t>
+          <t>https://www.acog.org/clinical/clinical-guidance/committee-opinion/articles/2020/04/physical-activity-and-exercise-during-pregnancy-and-the-postpartum-period</t>
         </is>
       </c>
     </row>
@@ -2958,7 +2985,7 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Postpartum Recovery: What to Expect</t>
+          <t>Returning to activity after childbirth</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -2968,7 +2995,7 @@
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_27)</t>
+          <t>Revised — WH_27; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -2978,32 +3005,32 @@
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>The 4th Trimester: Diastasis Recti, Pelvic Floor Healing &amp; Autonomic Rebalance</t>
+          <t>Returning to activity after childbirth</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>Tam Cá Nguyệt Thứ Tư: Phục Hồi Tách Cơ Bụng (Diastasis Recti), Sàn Chậu &amp; Sức Bền Thần Kinh</t>
+          <t>Trở lại vận động sau sinh: phục hồi theo triệu chứng</t>
         </is>
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>Hành trình làm mẹ không dừng lại ở phòng sinh; 12 tuần đầu tiên sau khi sinh—được y học gọi là 'Tam Cá Nguyệt Thứ Tư'—là giai đoạn cơ thể trải qua cú sốc tụt dốc hormone lớn nhất đời người cùng sự tái cấu trúc cơ bụng và sàn chậu. Khám phá cách chẩn đoán tách cơ bụng (Diastasis Recti) và phác đồ phục hồi thể lực an toàn.</t>
+          <t>Thời điểm trở lại tập tùy phương pháp sinh, biến chứng và cảm giác hồi phục.</t>
         </is>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>Đừng vội vàng gập bụng truyền thống (Crunches/Sit-ups) sau sinh vì chúng làm tăng áp lực ổ bụng và khiến vết tách cơ bụng hở rộng hơn. Hãy bắt đầu bằng các bài tập kích hoạt cơ ngang bụng sâu (Transversus Abdominis) qua nhịp thở cơ hoành, và cho phép hệ thần kinh 1–2 tuần để nhịp tim nghỉ ngơi hạ nhiệt tự nhiên.</t>
+          <t>Bắt đầu với hoạt động nhẹ, nghỉ đủ và tăng từng bước khi thấy thoải mái. Sau mổ lấy thai hoặc biến chứng, hỏi thời điểm phù hợp. Nhờ đánh giá nếu có rò tiểu, nặng vùng chậu hoặc đau trong các động tác.</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
         <is>
-          <t>HO-08 (Postpartum recovery: rapid HRV rebound and RHR normalization within 6-8 weeks - Rowan 2022)</t>
+          <t>Returning to activity after childbirth (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
-          <t>Dufour et al. (J Orthop Sports Phys Ther, 2019); Goom et al. (Br J Sports Med, 2019 - Returning to Running)</t>
+          <t>https://www.acog.org/womens-health/faqs/exercise-after-pregnancy</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3045,7 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>PCOS: Symptoms &amp; What You Should Know</t>
+          <t>PCOS/PMOS: diagnosis and comprehensive care</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -3028,7 +3055,7 @@
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_28)</t>
+          <t>Revised — WH_28; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -3038,32 +3065,32 @@
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>PCOS Demystified: Rotterdam Criteria, Hyperandrogenism &amp; Insulin Resistance</t>
+          <t>PCOS/PMOS: diagnosis and comprehensive care</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>Hội Chứng Buồng Trứng Đa Nang (PCOS): Tiêu Chuẩn Rotterdam &amp; Giải Pháp Kháng Insulin</t>
+          <t>PCOS/PMOS: chẩn đoán và chăm sóc vượt ra ngoài hình ảnh buồng trứng</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>PCOS không đơn thuần là sự xuất hiện của các nang nhỏ trên buồng trứng; đó là một hội chứng rối loạn chuyển hóa và nội tiết toàn thân phức tạp ảnh hưởng đến 1 trên 10 phụ nữ. Tìm hiểu tiêu chuẩn chẩn đoán Rotterdam quốc tế, vai trò cốt lõi của tình trạng kháng insulin và phác đồ tập luyện dinh dưỡng để phục hồi chu kỳ rụng trứng.</t>
+          <t>Tình trạng thường được biết là PCOS liên quan kinh nguyệt, androgen và sức khỏe chuyển hóa; không đơn thuần là có nang trên siêu âm.</t>
         </is>
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>Để chẩn đoán PCOS chuẩn xác, bạn cần thỏa mãn ít nhất 2 trong 3 tiêu chuẩn Rotterdam: kinh nguyệt thưa/vô kinh, dấu hiệu thừa androgen (rậm lông, mụn bọc, rụng tóc), hoặc hình ảnh đa nang trên siêu âm. Chìa khóa điều trị số 1 không phải là thuốc tránh thai mà là giải quyết tình trạng Kháng Insulin bằng tập tạ kháng lực và bổ sung Myo-Inositol.</t>
+          <t>Mang thông tin chu kỳ, triệu chứng và mục tiêu như điều hòa kinh hoặc có thai khi khám. Chăm sóc nên bao gồm sức khỏe chuyển hóa và tâm lý, vận động, dinh dưỡng cùng điều trị phù hợp, tránh phán xét dựa trên cân nặng.</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>HO-02 (Long/irregular cycles &gt;35-45 days), HO-04 (Lack of biphasic temperature shift in anovulatory cycles)</t>
+          <t>PCOS/PMOS: diagnosis and comprehensive care (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
-          <t>Teede et al. (Hum Reprod, International PCOS Guideline 2023); Rotterdam ESHRE/ASRM Consensus (2004)</t>
+          <t>https://www.monash.edu/medicine/mchri/pcos/guideline</t>
         </is>
       </c>
     </row>
@@ -3078,7 +3105,7 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Endometriosis: Understanding the Signs</t>
+          <t>Endometriosis: recognizing symptoms and seeking care</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -3088,7 +3115,7 @@
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_29)</t>
+          <t>Revised — WH_29; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -3098,32 +3125,32 @@
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Endometriosis Uncovered: Retrograde Menstruation, Chronic Inflammation &amp; Care</t>
+          <t>Endometriosis: recognizing symptoms and seeking care</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>Lạc Nội Mạc Tử Cung: Nhận Diện Cơn Đau Vùng Chậu Mãn Tính &amp; Lộ Trình Chẩn Đoán Sớm</t>
+          <t>Lạc nội mạc tử cung: đau nhiều cần được lắng nghe</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>Đau bụng kinh dữ dội đến mức ngất xỉu, nôn mửa hoặc phải nghỉ làm không bao giờ là chuyện 'bình thường'. Lạc nội mạc tử cung (Endometriosis) là một bệnh lý viêm mãn tính phức tạp hành hạ gần 200 triệu phụ nữ trên toàn cầu, với độ trễ chẩn đoán trung bình từ 7 đến 10 năm. Tìm hiểu cơ chế sinh học, dấu hiệu cảnh báo và lộ trình điều trị y khoa chuẩn mực.</t>
+          <t>Lạc nội mạc tử cung có thể gây đau vùng chậu, đau theo kỳ kinh, đau khi quan hệ hoặc khó có thai.</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>Nếu cơn đau bụng kinh của bạn không thuyên giảm khi dùng thuốc giảm đau NSAIDs thông thường, hoặc lan ra sau lưng, đau buốt khi đi vệ sinh hay khi quan hệ sâu, đừng chần chừ. Hãy tìm đến bác sĩ chuyên khoa sâu về Lạc nội mạc tử cung để siêu âm chuyên sâu hoặc phẫu thuật nội soi bóc tách tổn thương.</t>
+          <t>Ghi thời điểm đau, ảnh hưởng sinh hoạt, triệu chứng ruột hoặc bàng quang và cách giảm đau đã thử. Mang nhật ký khi khám; hỏi kế hoạch điều trị và theo dõi nếu triệu chứng còn ảnh hưởng dù đánh giá ban đầu chưa rõ.</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
         <is>
-          <t>HO-06 (Severe pain logs throughout cycle, not just day 1), REC-01 (Chronically depressed HRV from inflammation)</t>
+          <t>Endometriosis: recognizing symptoms and seeking care (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L33" s="7" t="inlineStr">
         <is>
-          <t>Zondervan et al. (Nat Rev Dis Primers, 2018); Giudice (NEJM, 2010); ESHRE Endometriosis Guideline (2022)</t>
+          <t>https://www.nhs.uk/conditions/endometriosis/</t>
         </is>
       </c>
     </row>
@@ -3138,7 +3165,7 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Perimenopause &amp; Menopause Explained</t>
+          <t>Perimenopause and menopause: symptoms and care</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -3148,7 +3175,7 @@
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>Completed (Written &amp; Published as WH_30)</t>
+          <t>Revised — WH_30; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -3158,36 +3185,2669 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>The Menopausal Transition: Vasomotor Fluctuations, Estrogen Cliff &amp; Bone Vitality</t>
+          <t>Perimenopause and menopause: symptoms and care</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>Tiền Mãn Kinh &amp; Mãn Kinh: Cơn Bốc Hỏa, Chuyển Dịch Nội Tiết &amp; Bảo Vệ Khung Xương</t>
+          <t>Tiền mãn kinh và mãn kinh: nhận biết và chọn cách chăm sóc</t>
         </is>
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>Thời kỳ tiền mãn kinh không phải là một công tắc bật tắt đột ngột ở tuổi 50; đó là một giai đoạn chuyển tiếp nội tiết kéo dài từ 4 đến 8 năm, bắt đầu từ độ tuổi ngoài 40 với những đợt sóng estrogen dao động dữ dội. Tìm hiểu tiêu chuẩn vàng STRAW+10, nguồn gốc các cơn bốc hỏa và chiến lược y học hiện đại để bước qua giai đoạn này với sức sống rạng ngời.</t>
+          <t>Chu kỳ thay đổi, bốc hỏa, khó ngủ và khô âm đạo có thể xuất hiện trong giai đoạn chuyển tiếp.</t>
         </is>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>Mãn kinh chỉ được xác định khi bạn đã mất kinh liên tục trọn vẹn 12 tháng. Trong giai đoạn tiền mãn kinh, hãy theo dõi sự dãn dài của chu kỳ (&gt; 7 ngày lệch chuẩn) trên thiết bị đeo, chủ động rèn luyện tạ kháng lực để chống mất xương và thảo luận sớm với bác sĩ về Liệu Pháp Hormone Mãn Kinh (MHT) trong 'Cửa Sổ Vàng' trước tuổi 60.</t>
+          <t>Ghi triệu chứng chính và mục tiêu điều trị. Duy trì vận động, dinh dưỡng và trao đổi về lựa chọn nội tiết hoặc không nội tiết với bác sĩ; quyết định dựa trên tiền sử, lợi ích, rủi ro và ưu tiên cá nhân.</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>HO-02 (Extreme cycle length variability), appleSleepingWristTemperature (nocturnal hot flash spikes), REC-01</t>
+          <t>Perimenopause and menopause: symptoms and care (educational topic; not a measured biomarker)</t>
         </is>
       </c>
       <c r="L34" s="7" t="inlineStr">
         <is>
-          <t>Harlow et al. (Menopause, STRAW+10 Staging System 2012); NAMS 2022 Hormone Therapy Position Statement</t>
+          <t>https://www.nhs.uk/conditions/menopause-and-perimenopause/symptoms/</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId30"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" style="1" min="1" max="1"/>
+    <col width="24" customWidth="1" style="1" min="2" max="2"/>
+    <col width="55" customWidth="1" style="1" min="3" max="3"/>
+    <col width="55" customWidth="1" style="1" min="4" max="4"/>
+    <col width="55" customWidth="1" style="1" min="5" max="5"/>
+    <col width="55" customWidth="1" style="1" min="6" max="6"/>
+    <col width="55" customWidth="1" style="1" min="7" max="7"/>
+    <col width="55" customWidth="1" style="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Content_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Title_VI</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Title_EN</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Source_Name</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Source_URL</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Public_URL</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>Review_Status</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>Limits_VI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="86" customHeight="1" s="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>LM_WH_01</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Chu kỳ kinh nguyệt: hiểu các giai đoạn mà không đóng khung bản thân</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>Understanding menstrual cycle phases</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Periods</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/periods/</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/LM_WH_01.html</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
+        <is>
+          <t>Năng lượng và tâm trạng có thể thay đổi nhưng không giống nhau ở mọi người. Thuốc nội tiết, sau sinh và tiền mãn kinh làm việc suy đoán pha từ lịch kém đáng tin hơn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="86" customHeight="1" s="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>LM_WH_02</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Dịch nhầy cổ tử cung: theo dõi thế nào cho hữu ích?</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Tracking cervical mucus usefully</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>ACOG — Fertility Awareness-Based Methods of Family Planning</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/womens-health/faqs/fertility-awareness-based-methods-of-family-planning</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/LM_WH_02.html</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>Ứng dụng ghi dịch tiết không tự trở thành phương pháp tránh thai đã được xác thực. Màu hoặc độ đặc riêng lẻ cũng không đủ chẩn đoán nhiễm trùng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="86" customHeight="1" s="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>LM_WH_03</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>BBT và nhiệt độ da: gợi ý rụng trứng, không xác nhận thai</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>BBT and skin temperature: understanding the limits</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>ACOG — Fertility Awareness-Based Methods of Family Planning</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/womens-health/faqs/fertility-awareness-based-methods-of-family-planning</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/LM_WH_03.html</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Nhiệt tăng chủ yếu gợi ý rụng trứng đã xảy ra, không dự báo chắc thời điểm sắp rụng. Không áp quy tắc BBT trực tiếp cho mọi cảm biến da hoặc dùng một chuỗi nhiệt cao để xác nhận thai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="86" customHeight="1" s="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>DM_WH_01</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Tập theo chu kỳ: ưu tiên triệu chứng hơn lịch pha cố định</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Cycle-aware training without rigid phase rules</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>McNulty et al. (2020) — The Effects of Menstrual Cycle Phase on Exercise Performance in Eumenorrheic Women</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/32661839/</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/DM_WH_01.html</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Theo dõi triệu chứng không đồng nghĩa đo được estrogen hoặc progesterone. Nghiên cứu ở người có chu kỳ tự nhiên không tự áp dụng cho người dùng tránh thai nội tiết.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="86" customHeight="1" s="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>DM_WH_02</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Cửa sổ thụ thai: dùng dự đoán với mức chắc chắn phù hợp</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>The fertile window and prediction uncertainty</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>ACOG — Fertility Awareness-Based Methods of Family Planning</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/womens-health/faqs/fertility-awareness-based-methods-of-family-planning</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/DM_WH_02.html</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Khoảng sáu ngày là mô hình sinh học, không phải lịch tránh thai an toàn do app tự tính. Dự đoán từ lịch và cảm biến không bảo đảm xác định mọi ngày có khả năng thụ thai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="86" customHeight="1" s="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>DM_WH_03</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>PMS, đau bụng kinh và thèm ăn: chăm sóc theo triệu chứng</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>PMS, cramps and appetite changes</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>NHS — PMS (premenstrual syndrome)</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/pre-menstrual-syndrome/</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/DM_WH_03.html</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Không cần chế độ ăn theo pha bắt buộc hay tự bổ sung liều cao để cân bằng hormone. Thèm ăn không đủ để suy ra thiếu một vi chất cụ thể.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="86" customHeight="1" s="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>WH_04</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Kinh nguyệt không đều: ghi nhận gì và khi nào đi khám?</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Irregular periods: tracking and seeking care</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Missed or late periods</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/symptoms/missed-or-late-periods/</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_04.html</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Khoảng chu kỳ trên dân số không phải ngưỡng chẩn đoán duy nhất. Thiết bị đeo không phân biệt được mọi nguyên nhân trễ kinh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="86" customHeight="1" s="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>WH_06</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Estrogen và progesterone: vai trò và giới hạn tự theo dõi</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Estrogen and progesterone: roles and tracking limits</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Endocrine Society — Reproductive Hormones</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>https://www.endocrine.org/patient-engagement/endocrine-library/hormones-and-endocrine-function/reproductive-hormones</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_06.html</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Đường cong trong sách là mô hình đơn giản, không phải kết quả xét nghiệm của bạn. HRV, nhịp tim và nhiệt độ da không đo trực tiếp estrogen hay progesterone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="86" customHeight="1" s="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>WH_07</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Tập trung và cảm xúc quanh kỳ kinh: theo dõi trải nghiệm thực tế</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Concentration and mood around your period</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>NHS — PMS (premenstrual syndrome)</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/pre-menstrual-syndrome/</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_07.html</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>Tương quan theo chu kỳ không chứng minh hormone là nguyên nhân duy nhất. Nhật ký hỗ trợ trao đổi, không chẩn đoán rối loạn hormone hay bệnh tâm lý.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="86" customHeight="1" s="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>WH_09</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Ham muốn nữ giới: nhiều yếu tố cùng góp phần</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Understanding sexual desire in women</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Low sex drive (loss of libido)</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/symptoms/loss-of-libido/</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_09.html</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Không có tần suất chuẩn áp dụng cho mọi người. Không dùng nhiệt độ, HRV hay ngày rụng trứng dự đoán để suy ra bạn phải có ham muốn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="86" customHeight="1" s="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>WH_10</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Cảm xúc theo chu kỳ: không phải ai cũng có đỉnh hưng phấn lúc rụng trứng</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Cycle-related mood changes without fixed peaks</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>NHS — PMS (premenstrual syndrome)</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/pre-menstrual-syndrome/</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_10.html</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Dự đoán của app không đọc được serotonin hay xác định ngày sẽ vui hoặc buồn. Không quy mọi triệu chứng tâm lý cho chu kỳ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="86" customHeight="1" s="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>WH_11</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Dịch tiết âm đạo và pH: dấu hiệu nào đáng chú ý?</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Vaginal discharge and pH: useful signs and limits</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>ACOG — Vulvovaginal Health</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/womens-health/faqs/vulvovaginal-health</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_11.html</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Que thử pH và ảnh chụp dịch tiết không thay thế thăm khám hoặc xét nghiệm khi cần. Không phải mọi hệ vi sinh khác mẫu sách đều là bệnh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="86" customHeight="1" s="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>WH_12</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Đau khi quan hệ: không cần cố chịu đựng</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Pain during sex: finding the cause</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>ACOG — When Sex Is Painful</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/womens-health/faqs/when-sex-is-painful</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_12.html</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Không mặc định đau là thiếu estrogen hoặc cơ yếu cần Kegel. Điều trị phụ thuộc nguyên nhân; chất bôi trơn hỗ trợ thoải mái nhưng không chữa mọi bệnh lý.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="86" customHeight="1" s="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>WH_13</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Sàn chậu nữ: sức mạnh cần đi cùng khả năng thả lỏng</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Pelvic-floor function in women</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Urinary incontinence: non-surgical treatment</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/urinary-incontinence/treatment/</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_13.html</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>Không dùng cảm giác siết mạnh hay số lần tập để suy ra mức cải thiện. Kegel không phải giải pháp chung cho đau khi quan hệ hoặc mọi rối loạn sàn chậu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="86" customHeight="1" s="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>WH_15</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Tập khi có kinh: chọn cường độ theo mức dễ chịu</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Exercising during your period</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>McNulty et al. (2020) — The Effects of Menstrual Cycle Phase on Exercise Performance in Eumenorrheic Women</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/32661839/</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_15.html</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>Không khẳng định một bài tập tăng tưới máu tử cung sẽ điều trị đau. Lịch pha do app dự đoán không thay trải nghiệm thực tế.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="86" customHeight="1" s="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>WH_16</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>HRV thay đổi theo chu kỳ: so với nền riêng của bạn</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>HRV changes across the menstrual cycle</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Schmalenberger et al. (2019) — A Systematic Review and Meta-Analysis of Within-Person Changes in Cardiac Vagal Activity across the Menstrual Cycle</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/31726666/</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_16.html</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>HRV không đo trực tiếp progesterone và không xác nhận rụng trứng. Một tỷ lệ giảm cố định cho mọi phụ nữ là diễn giải quá mức.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="86" customHeight="1" s="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>WH_17</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Tập sức mạnh cho nữ: xây thói quen lâu dài</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Strength training for women</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>WHO — Physical activity</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>https://www.who.int/news-room/fact-sheets/detail/physical-activity</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_17.html</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Bằng chứng hiện tại không buộc phải dồn tập sức mạnh vào một pha chu kỳ. Lợi ích không được bảo đảm chỉ bằng tăng số cân hoặc điểm Strain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="86" customHeight="1" s="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>WH_18</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>REDs: khi ăn không đủ so với nhu cầu tập luyện</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>REDs and low energy availability</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Mountjoy et al. (2023) — IOC consensus statement on Relative Energy Deficiency in Sport (REDs)</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>https://bjsm.bmj.com/content/57/17/1073</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_18.html</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Không có một ngưỡng calo từ đồng hồ chẩn đoán REDs cho tất cả. Ước tính tiêu hao và năng lượng ăn vào đều có sai số; cần đánh giá nhiều mặt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="86" customHeight="1" s="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>WH_19</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Khó ngủ trước kỳ kinh: chăm sóc triệu chứng, không chạy theo REM</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Sleep difficulties before your period</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>NHS — PMS (premenstrual syndrome)</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/pre-menstrual-syndrome/</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_19.html</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>Không có nhiệt độ phòng duy nhất phù hợp mọi người hoặc lời hứa làm mát sẽ khôi phục REM. Các giai đoạn trên thiết bị đeo vẫn là ước tính.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="86" customHeight="1" s="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>WH_20</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Stress và trễ kinh: cần xem xét những nguyên nhân nào?</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Stress and a late period: considering other causes</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Missed or late periods</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/symptoms/missed-or-late-periods/</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_20.html</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>Nhịp tim hoặc HRV không đo được nồng độ cortisol và không phân biệt mọi nguyên nhân mất kinh. Tự bổ sung sản phẩm giảm cortisol có thể làm chậm đánh giá đúng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="86" customHeight="1" s="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>WH_21</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Dinh dưỡng quanh chu kỳ: đủ năng lượng trước khi theo thực đơn theo pha</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Nutrition across the cycle</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>WHO — Healthy diet</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>https://www.who.int/news-room/fact-sheets/detail/healthy-diet</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_21.html</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>Không gán cơn thèm một món cho thiếu khoáng chất cụ thể. Không hứa seed cycling hay thực phẩm giải độc estrogen sẽ cân bằng nội tiết.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="86" customHeight="1" s="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>WH_22</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Kinh nhiều và thiếu sắt: xét nghiệm trước khi tự bổ sung</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Heavy periods and iron deficiency</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Heavy periods</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/heavy-periods/</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_22.html</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>Không tự chẩn đoán thiếu sắt từ triệu chứng hoặc dùng một mức ferritin tối ưu cho tất cả. Liều và thời gian bổ sung phụ thuộc kết quả và bối cảnh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="86" customHeight="1" s="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>WH_23</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Canh thời điểm thụ thai: giảm áp lực phải đúng một ngày</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Timing intercourse when trying to conceive</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>ASRM (2022) — Optimizing natural fertility: a committee opinion</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>https://integration.asrm.org/globalassets/_asrm/practice-guidance/practice-guidelines/pdf/optimizing_natural_fertility.pdf</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_23.html</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>Một biểu đồ xác suất nghiên cứu không phải dự báo cá nhân. Theo dõi không bảo đảm có thai và không thay đánh giá chất lượng tinh trùng hay các yếu tố sinh sản khác.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="86" customHeight="1" s="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>WH_24</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Dấu hiệu thai sớm: dùng que thử thay vì suy từ thiết bị đeo</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Early pregnancy signs and reliable testing</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Doing a pregnancy test</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/pregnancy/trying-for-a-baby/doing-a-pregnancy-test/</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_24.html</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>Không gọi biến động nhiệt là dấu hiệu làm tổ chắc chắn. Chảy máu ít cũng không đủ để phân biệt thai bình thường, kinh hay vấn đề cần khám.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="86" customHeight="1" s="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>WH_25</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Cơ thể thay đổi khi mang thai: theo dõi triệu chứng quan trọng</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Body changes during pregnancy</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Common health problems in pregnancy</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/pregnancy/common-symptoms/common-health-problems/</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_25.html</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>Dữ liệu người không mang thai không tự áp dụng cho thai kỳ. Không có một ngưỡng đồng hồ bảo đảm thai bình thường ở mọi người.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="86" customHeight="1" s="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>WH_26</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Vận động trong thai kỳ: trao đổi trước và theo dõi dấu hiệu dừng</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Exercise during pregnancy</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>ACOG (2020) — Physical Activity and Exercise During Pregnancy and the Postpartum Period</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/clinical/clinical-guidance/committee-opinion/articles/2020/04/physical-activity-and-exercise-during-pregnancy-and-the-postpartum-period</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_26.html</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>Không có giới hạn 140 nhịp/phút áp dụng cho tất cả. Mục tiêu chung không vượt qua chỉ định hạn chế tập nếu có biến chứng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="86" customHeight="1" s="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>WH_27</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Trở lại vận động sau sinh: phục hồi theo triệu chứng</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Returning to activity after childbirth</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>ACOG — Exercise After Pregnancy</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/womens-health/faqs/exercise-after-pregnancy</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_27.html</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>Mốc sáu tuần không tự là giấy phép chạy nhảy hay tập nặng. Không hứa một bài tập đóng hoàn toàn khe cơ bụng hoặc phục hồi theo số ngày cố định.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="86" customHeight="1" s="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>WH_28</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>PCOS/PMOS: chẩn đoán và chăm sóc vượt ra ngoài hình ảnh buồng trứng</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>PCOS/PMOS: diagnosis and comprehensive care</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>Monash University — International evidence-based PCOS / PMOS guideline</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>https://www.monash.edu/medicine/mchri/pcos/guideline</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_28.html</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>Tiêu chuẩn ở người trưởng thành và vị thành niên khác nhau. Không tự chẩn đoán bằng một tỷ lệ LH/FSH, chỉ số insulin hoặc dự đoán app; không có chế độ ăn chữa khỏi cho tất cả.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="86" customHeight="1" s="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>WH_29</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Lạc nội mạc tử cung: đau nhiều cần được lắng nghe</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Endometriosis: recognizing symptoms and seeking care</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Endometriosis</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/endometriosis/</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_29.html</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>Một kết quả kiểm tra ban đầu bình thường không giải thích được mọi cơn đau. Không có dữ liệu từ HRV hoặc app chu kỳ chẩn đoán hay loại trừ bệnh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="86" customHeight="1" s="1">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>WH_30</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Tiền mãn kinh và mãn kinh: nhận biết và chọn cách chăm sóc</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Perimenopause and menopause: symptoms and care</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Symptoms of menopause and perimenopause</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/menopause-and-perimenopause/symptoms/</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>https://test-repo-y1wb.onrender.com/posts/WH_30.html</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>Revised against cited sources; clinical sign-off not recorded</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>Không dùng nhiệt độ da hay một kết quả hormone đơn lẻ để tự xác nhận giai đoạn. Thảo dược hoặc sản phẩm cân bằng hormone không được mặc định hiệu quả và an toàn.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H31"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId60"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" style="1" min="1" max="1"/>
+    <col width="24" customWidth="1" style="1" min="2" max="2"/>
+    <col width="55" customWidth="1" style="1" min="3" max="3"/>
+    <col width="55" customWidth="1" style="1" min="4" max="4"/>
+    <col width="55" customWidth="1" style="1" min="5" max="5"/>
+    <col width="55" customWidth="1" style="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Source_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Supports_VI</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Supports_EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="86" customHeight="1" s="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>periods</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Periods</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/periods/</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>Chu kỳ, triệu chứng và chảy máu bất thường</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>Cycles, symptoms and abnormal bleeding</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="86" customHeight="1" s="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>fertility</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>ACOG — Fertility Awareness-Based Methods of Family Planning</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/womens-health/faqs/fertility-awareness-based-methods-of-family-planning</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Professional patient guidance</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Chất nhầy, BBT, thời điểm sinh sản và giới hạn tránh thai</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>Mucus, BBT, fertile timing and contraceptive limitations</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="86" customHeight="1" s="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>missed</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Missed or late periods</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/symptoms/missed-or-late-periods/</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Nguyên nhân trễ kinh và thời điểm đi khám</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Causes of missed periods and when to seek care</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="86" customHeight="1" s="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>vaginal</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>ACOG — Vulvovaginal Health</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/womens-health/faqs/vulvovaginal-health</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Professional patient guidance</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Vệ sinh vùng kín, dịch tiết, thay đổi niêm mạc và điều trị</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Vulvovaginal care, discharge, tissue changes and treatments</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="86" customHeight="1" s="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>test_pregnancy</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Doing a pregnancy test</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/pregnancy/trying-for-a-baby/doing-a-pregnancy-test/</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Thời điểm thử thai và xử trí kết quả âm tính sớm</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>Pregnancy test timing and early negative results</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="86" customHeight="1" s="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>cycle_training</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>McNulty et al. (2020) — The Effects of Menstrual Cycle Phase on Exercise Performance in Eumenorrheic Women</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/32661839/</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Hiệu ứng trung bình nhỏ, chất lượng bằng chứng thấp; cần cá nhân hóa</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Small average effects and low-quality evidence; individualized approach</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="86" customHeight="1" s="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>strength_cycle</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Colenso-Semple et al. (2023) — Current evidence shows no influence of women's menstrual cycle phase on acute strength performance or adaptations to resistance exercise training</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/37033884/</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Umbrella review</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Chưa đủ cơ sở kê lịch tập sức mạnh cố định theo pha</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Insufficient basis for fixed phase-based resistance programming</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="86" customHeight="1" s="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>reds</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Mountjoy et al. (2023) — IOC consensus statement on Relative Energy Deficiency in Sport (REDs)</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>https://bjsm.bmj.com/content/57/17/1073</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Consensus statement</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Thiếu năng lượng, xương, kinh nguyệt và đánh giá đa chuyên ngành</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Low energy availability, bone, menstrual health and multidisciplinary assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="86" customHeight="1" s="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>pms</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>NHS — PMS (premenstrual syndrome)</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/pre-menstrual-syndrome/</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Triệu chứng PMS, nhật ký và lựa chọn chăm sóc</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>PMS symptoms, symptom diaries and care options</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="86" customHeight="1" s="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>diet</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>WHO — Healthy diet</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>https://www.who.int/news-room/fact-sheets/detail/healthy-diet</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Chế độ ăn đa dạng và chất lượng thực phẩm</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Dietary variety and food quality</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="86" customHeight="1" s="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>reproductive_hormones</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Endocrine Society — Reproductive Hormones</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>https://www.endocrine.org/patient-engagement/endocrine-library/hormones-and-endocrine-function/reproductive-hormones</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Professional patient guidance</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Vai trò các hormone sinh sản và xét nghiệm phù hợp</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Reproductive hormone roles and appropriate testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="86" customHeight="1" s="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>menopause</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Symptoms of menopause and perimenopause</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/menopause-and-perimenopause/symptoms/</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Triệu chứng tiền mãn kinh và mãn kinh; khi cần khám</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>Perimenopause and menopause symptoms; seeking care</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="86" customHeight="1" s="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>libido</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Low sex drive (loss of libido)</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/symptoms/loss-of-libido/</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Nhiều yếu tố ảnh hưởng ham muốn và chăm sóc theo nguyên nhân</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>Multiple influences on desire and cause-based care</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="86" customHeight="1" s="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>pain_sex</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>ACOG — When Sex Is Painful</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/womens-health/faqs/when-sex-is-painful</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Professional patient guidance</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Nguyên nhân đau khi quan hệ và tiếp cận chăm sóc</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>Causes and care of painful sex</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="86" customHeight="1" s="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>sexual_health</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Devon Sexual Health (NHS) — Relationships and intimacy</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>https://www.devonsexualhealth.nhs.uk/your-sexual-health/relationships-and-intimacy/</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Sexual health service guidance</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Đồng thuận, thân mật và thủ dâm</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Consent, intimacy and masturbation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="86" customHeight="1" s="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>pelvic_women</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Urinary incontinence: non-surgical treatment</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/urinary-incontinence/treatment/</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Đánh giá sàn chậu và tập có giám sát cho rò tiểu</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>Pelvic-floor assessment and supervised training for leakage</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="86" customHeight="1" s="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>pelvic_women_relax</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Cambridge University Hospitals — Female pelvic floor muscle exercises</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>https://www.cuh.nhs.uk/patient-information/female-pelvic-floor-muscle-exercises/</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Physiotherapy patient guidance</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Cần thả lỏng đầy đủ giữa các lần co cơ</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Full relaxation between pelvic-floor contractions</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="86" customHeight="1" s="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>heavy</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Heavy periods</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/heavy-periods/</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Nhận biết chảy máu nhiều và các hướng điều trị</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Recognizing heavy menstrual bleeding and treatment options</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="86" customHeight="1" s="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>cycle_hrv</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Schmalenberger et al. (2019) — A Systematic Review and Meta-Analysis of Within-Person Changes in Cardiac Vagal Activity across the Menstrual Cycle</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/31726666/</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Biến đổi hoạt động phế vị theo chu kỳ ở cấp độ nhóm</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Group-level cycle-related changes in cardiac vagal activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="86" customHeight="1" s="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>hrv</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Shaffer &amp; Ginsberg (2017) — An Overview of Heart Rate Variability Metrics and Norms</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/29034226/</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>Narrative review</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Chỉ số HRV, bối cảnh đo và giới hạn so sánh</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>HRV metrics, recording context and comparability limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="86" customHeight="1" s="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>pulse</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>American Heart Association — All About Heart Rate</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>https://www.heart.org/en/health-topics/high-blood-pressure/the-facts-about-high-blood-pressure/all-about-heart-rate-pulse</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>Professional patient guidance</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>Nhịp tim nghỉ, yếu tố ảnh hưởng và triệu chứng cần khám</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Resting pulse, influencing factors and warning symptoms</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="86" customHeight="1" s="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>activity</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>WHO — Physical activity</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>https://www.who.int/news-room/fact-sheets/detail/physical-activity</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>Public health guideline summary</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Khuyến nghị vận động theo nhóm đối tượng</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Activity recommendations by population</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="86" customHeight="1" s="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>overtraining</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Meeusen et al. (2013) — Prevention, diagnosis, and treatment of the overtraining syndrome</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/23247672/</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>Joint consensus statement</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>Quá tải, chẩn đoán loại trừ và thiếu chỉ dấu đơn lẻ</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Overtraining, exclusion diagnosis and absence of a single marker</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="86" customHeight="1" s="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>sleep_habits</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>NHLBI — Healthy Sleep Habits</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhlbi.nih.gov/health/sleep-deprivation/healthy-sleep-habits</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Thói quen ngủ và lịch sinh hoạt</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Sleep habits and consistent schedules</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="86" customHeight="1" s="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>sleep_tech</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Schutte-Rodin et al. (2021) — Evaluating consumer and clinical sleep technologies: an American Academy of Sleep Medicine update</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/34314344/</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>Professional society review</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Giới hạn đánh giá và xác thực công nghệ theo dõi giấc ngủ</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>Evaluation and validation limits of sleep technologies</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="86" customHeight="1" s="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>iron</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Iron deficiency anaemia</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/iron-deficiency-anaemia/</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Xét nghiệm thiếu máu và bổ sung sắt theo đánh giá</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>Anaemia testing and assessed iron replacement</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="86" customHeight="1" s="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>natural_fertility</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>ASRM (2022) — Optimizing natural fertility: a committee opinion</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>https://integration.asrm.org/globalassets/_asrm/practice-guidance/practice-guidelines/pdf/optimizing_natural_fertility.pdf</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Committee opinion</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Thời điểm quan hệ, giới hạn dự đoán và khi đánh giá hiếm muộn</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>Intercourse timing, prediction limitations and fertility evaluation</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="86" customHeight="1" s="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>ectopic</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Ectopic pregnancy: symptoms</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/ectopic-pregnancy/symptoms/</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>Đau bụng, chảy máu, đau vai và chăm sóc khẩn</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>Pain, bleeding, shoulder pain and urgent care</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="86" customHeight="1" s="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>pregnancy</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Common health problems in pregnancy</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/pregnancy/common-symptoms/common-health-problems/</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Triệu chứng thường gặp trong thai kỳ</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>Common pregnancy symptoms</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="86" customHeight="1" s="1">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>pregnancy_exercise</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>ACOG (2020) — Physical Activity and Exercise During Pregnancy and the Postpartum Period</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/clinical/clinical-guidance/committee-opinion/articles/2020/04/physical-activity-and-exercise-during-pregnancy-and-the-postpartum-period</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Committee guidance</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>Vận động thai kỳ, cá nhân hóa và dấu hiệu dừng tập</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Pregnancy activity, individualization and exercise warning signs</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="86" customHeight="1" s="1">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>intensity</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>CDC — Measuring Physical Activity Intensity</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/physicalactivity/basics/measuring/index.html</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Talk test phân biệt vận động vừa và mạnh</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>Talk test for moderate and vigorous activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="86" customHeight="1" s="1">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>postpartum</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>ACOG — Exercise After Pregnancy</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/womens-health/faqs/exercise-after-pregnancy</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Professional patient guidance</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>Trở lại vận động sau sinh tùy phương pháp sinh và biến chứng</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>Postpartum return to activity by delivery and complications</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="86" customHeight="1" s="1">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>pcos</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>Monash University — International evidence-based PCOS / PMOS guideline</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>https://www.monash.edu/medicine/mchri/pcos/guideline</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>International guideline</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>Chẩn đoán và chăm sóc toàn diện; cập nhật tên PMOS năm 2026</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>Diagnosis and comprehensive care; PMOS terminology update in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="86" customHeight="1" s="1">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>endometriosis</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Endometriosis</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/endometriosis/</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>Triệu chứng, chẩn đoán và điều trị lạc nội mạc tử cung</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>Endometriosis symptoms, assessment and treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="86" customHeight="1" s="1">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>menopause_care</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Menopause and perimenopause: treatment</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/menopause-and-perimenopause/treatment/</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>Thảo luận lợi ích và rủi ro điều trị triệu chứng mãn kinh</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>Discussing benefits and risks of menopause symptom treatment</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F36"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId35"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(content): develop original outlines into in-depth evidence-based articles
</commit_message>
<xml_diff>
--- a/docs/Master_Health_Articles_MVP - 30 Blog Topics.xlsx
+++ b/docs/Master_Health_Articles_MVP - 30 Blog Topics.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Reviewed_Content'!$A$1:$H$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source_Register'!$A$1:$F$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source_Register'!$A$1:$F$52</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="G3" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H3" s="10" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H4" s="10" t="inlineStr">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H5" s="10" t="inlineStr">
@@ -3513,7 +3513,7 @@
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H7" s="10" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H8" s="10" t="inlineStr">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H9" s="10" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
@@ -3723,7 +3723,7 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H14" s="10" t="inlineStr">
@@ -3891,7 +3891,7 @@
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H17" s="10" t="inlineStr">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
@@ -4059,7 +4059,7 @@
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H19" s="10" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
@@ -4143,7 +4143,7 @@
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H21" s="10" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H22" s="10" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H23" s="10" t="inlineStr">
@@ -4269,7 +4269,7 @@
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H24" s="10" t="inlineStr">
@@ -4311,7 +4311,7 @@
       </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H25" s="10" t="inlineStr">
@@ -4353,7 +4353,7 @@
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H26" s="10" t="inlineStr">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H27" s="10" t="inlineStr">
@@ -4437,7 +4437,7 @@
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H28" s="10" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H29" s="10" t="inlineStr">
@@ -4521,7 +4521,7 @@
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H30" s="10" t="inlineStr">
@@ -4563,7 +4563,7 @@
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>Revised against cited sources; clinical sign-off not recorded</t>
+          <t>Long-form development of original outline; sources checked; clinical sign-off not recorded</t>
         </is>
       </c>
       <c r="H31" s="10" t="inlineStr">
@@ -4646,7 +4646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="1" min="1" max="1"/>
@@ -4788,17 +4788,17 @@
     <row r="5" ht="86" customHeight="1" s="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>vaginal</t>
+          <t>reproductive_hormones</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>ACOG — Vulvovaginal Health</t>
+          <t>Endocrine Society — Reproductive Hormones</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>https://www.acog.org/womens-health/faqs/vulvovaginal-health</t>
+          <t>https://www.endocrine.org/patient-engagement/endocrine-library/hormones-and-endocrine-function/reproductive-hormones</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -4808,221 +4808,221 @@
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>Vệ sinh vùng kín, dịch tiết, thay đổi niêm mạc và điều trị</t>
+          <t>Vai trò các hormone sinh sản và xét nghiệm phù hợp</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>Vulvovaginal care, discharge, tissue changes and treatments</t>
+          <t>Reproductive hormone roles and appropriate testing</t>
         </is>
       </c>
     </row>
     <row r="6" ht="86" customHeight="1" s="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>test_pregnancy</t>
+          <t>openstax_cycle</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>NHS — Doing a pregnancy test</t>
+          <t>OpenStax Biology 2e — Hormonal Control of Human Reproduction</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>https://www.nhs.uk/pregnancy/trying-for-a-baby/doing-a-pregnancy-test/</t>
+          <t>https://openstax.org/books/biology-2e/pages/43-4-hormonal-control-of-human-reproduction</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Public health guidance</t>
+          <t>Physiology textbook</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Thời điểm thử thai và xử trí kết quả âm tính sớm</t>
+          <t>FSH, LH, hormone buồng trứng và trình tự sinh lý chu kỳ</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Pregnancy test timing and early negative results</t>
+          <t>FSH, LH, ovarian hormones and the physiological cycle sequence</t>
         </is>
       </c>
     </row>
     <row r="7" ht="86" customHeight="1" s="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>cycle_training</t>
+          <t>test_pregnancy</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>McNulty et al. (2020) — The Effects of Menstrual Cycle Phase on Exercise Performance in Eumenorrheic Women</t>
+          <t>NHS — Doing a pregnancy test</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/32661839/</t>
+          <t>https://www.nhs.uk/pregnancy/trying-for-a-baby/doing-a-pregnancy-test/</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Systematic review and meta-analysis</t>
+          <t>Public health guidance</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>Hiệu ứng trung bình nhỏ, chất lượng bằng chứng thấp; cần cá nhân hóa</t>
+          <t>Thời điểm thử thai và xử trí kết quả âm tính sớm</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>Small average effects and low-quality evidence; individualized approach</t>
+          <t>Pregnancy test timing and early negative results</t>
         </is>
       </c>
     </row>
     <row r="8" ht="86" customHeight="1" s="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>strength_cycle</t>
+          <t>ectopic</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Colenso-Semple et al. (2023) — Current evidence shows no influence of women's menstrual cycle phase on acute strength performance or adaptations to resistance exercise training</t>
+          <t>NHS — Ectopic pregnancy: symptoms</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/37033884/</t>
+          <t>https://www.nhs.uk/conditions/ectopic-pregnancy/symptoms/</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Umbrella review</t>
+          <t>Public health guidance</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>Chưa đủ cơ sở kê lịch tập sức mạnh cố định theo pha</t>
+          <t>Đau bụng, chảy máu, đau vai và chăm sóc khẩn</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Insufficient basis for fixed phase-based resistance programming</t>
+          <t>Pain, bleeding, shoulder pain and urgent care</t>
         </is>
       </c>
     </row>
     <row r="9" ht="86" customHeight="1" s="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>reds</t>
+          <t>cycle_training</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Mountjoy et al. (2023) — IOC consensus statement on Relative Energy Deficiency in Sport (REDs)</t>
+          <t>McNulty et al. (2020) — The Effects of Menstrual Cycle Phase on Exercise Performance in Eumenorrheic Women</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>https://bjsm.bmj.com/content/57/17/1073</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/32661839/</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Consensus statement</t>
+          <t>Systematic review and meta-analysis</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Thiếu năng lượng, xương, kinh nguyệt và đánh giá đa chuyên ngành</t>
+          <t>Hiệu ứng trung bình nhỏ, chất lượng bằng chứng thấp; cần cá nhân hóa</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>Low energy availability, bone, menstrual health and multidisciplinary assessment</t>
+          <t>Small average effects and low-quality evidence; individualized approach</t>
         </is>
       </c>
     </row>
     <row r="10" ht="86" customHeight="1" s="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>pms</t>
+          <t>strength_cycle</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>NHS — PMS (premenstrual syndrome)</t>
+          <t>Colenso-Semple et al. (2023) — Current evidence shows no influence of women's menstrual cycle phase on acute strength performance or adaptations to resistance exercise training</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>https://www.nhs.uk/conditions/pre-menstrual-syndrome/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/37033884/</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Public health guidance</t>
+          <t>Umbrella review</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>Triệu chứng PMS, nhật ký và lựa chọn chăm sóc</t>
+          <t>Chưa đủ cơ sở kê lịch tập sức mạnh cố định theo pha</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>PMS symptoms, symptom diaries and care options</t>
+          <t>Insufficient basis for fixed phase-based resistance programming</t>
         </is>
       </c>
     </row>
     <row r="11" ht="86" customHeight="1" s="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>diet</t>
+          <t>vaginal</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>WHO — Healthy diet</t>
+          <t>ACOG — Vulvovaginal Health</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>https://www.who.int/news-room/fact-sheets/detail/healthy-diet</t>
+          <t>https://www.acog.org/womens-health/faqs/vulvovaginal-health</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Public health guidance</t>
+          <t>Professional patient guidance</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>Chế độ ăn đa dạng và chất lượng thực phẩm</t>
+          <t>Vệ sinh vùng kín, dịch tiết, thay đổi niêm mạc và điều trị</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>Dietary variety and food quality</t>
+          <t>Vulvovaginal care, discharge, tissue changes and treatments</t>
         </is>
       </c>
     </row>
     <row r="12" ht="86" customHeight="1" s="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>reproductive_hormones</t>
+          <t>pain_sex</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Endocrine Society — Reproductive Hormones</t>
+          <t>ACOG — When Sex Is Painful</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>https://www.endocrine.org/patient-engagement/endocrine-library/hormones-and-endocrine-function/reproductive-hormones</t>
+          <t>https://www.acog.org/womens-health/faqs/when-sex-is-painful</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -5032,61 +5032,61 @@
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>Vai trò các hormone sinh sản và xét nghiệm phù hợp</t>
+          <t>Nguyên nhân đau khi quan hệ và tiếp cận chăm sóc</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>Reproductive hormone roles and appropriate testing</t>
+          <t>Causes and care of painful sex</t>
         </is>
       </c>
     </row>
     <row r="13" ht="86" customHeight="1" s="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>menopause</t>
+          <t>reds</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>NHS — Symptoms of menopause and perimenopause</t>
+          <t>Mountjoy et al. (2023) — IOC consensus statement on Relative Energy Deficiency in Sport (REDs)</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>https://www.nhs.uk/conditions/menopause-and-perimenopause/symptoms/</t>
+          <t>https://bjsm.bmj.com/content/57/17/1073</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Public health guidance</t>
+          <t>Consensus statement</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>Triệu chứng tiền mãn kinh và mãn kinh; khi cần khám</t>
+          <t>Thiếu năng lượng, xương, kinh nguyệt và đánh giá đa chuyên ngành</t>
         </is>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Perimenopause and menopause symptoms; seeking care</t>
+          <t>Low energy availability, bone, menstrual health and multidisciplinary assessment</t>
         </is>
       </c>
     </row>
     <row r="14" ht="86" customHeight="1" s="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>libido</t>
+          <t>pms</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>NHS — Low sex drive (loss of libido)</t>
+          <t>NHS — PMS (premenstrual syndrome)</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>https://www.nhs.uk/symptoms/loss-of-libido/</t>
+          <t>https://www.nhs.uk/conditions/pre-menstrual-syndrome/</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -5096,93 +5096,93 @@
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>Nhiều yếu tố ảnh hưởng ham muốn và chăm sóc theo nguyên nhân</t>
+          <t>Triệu chứng PMS, nhật ký và lựa chọn chăm sóc</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>Multiple influences on desire and cause-based care</t>
+          <t>PMS symptoms, symptom diaries and care options</t>
         </is>
       </c>
     </row>
     <row r="15" ht="86" customHeight="1" s="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>pain_sex</t>
+          <t>diet</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>ACOG — When Sex Is Painful</t>
+          <t>WHO — Healthy diet</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>https://www.acog.org/womens-health/faqs/when-sex-is-painful</t>
+          <t>https://www.who.int/news-room/fact-sheets/detail/healthy-diet</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>Professional patient guidance</t>
+          <t>Public health guidance</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Nguyên nhân đau khi quan hệ và tiếp cận chăm sóc</t>
+          <t>Chế độ ăn đa dạng và chất lượng thực phẩm</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Causes and care of painful sex</t>
+          <t>Dietary variety and food quality</t>
         </is>
       </c>
     </row>
     <row r="16" ht="86" customHeight="1" s="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>sexual_health</t>
+          <t>sleep_clock</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Devon Sexual Health (NHS) — Relationships and intimacy</t>
+          <t>NHLBI — Your Sleep/Wake Cycle</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>https://www.devonsexualhealth.nhs.uk/your-sexual-health/relationships-and-intimacy/</t>
+          <t>https://www.nhlbi.nih.gov/health/sleep/sleep-wake-cycle</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>Sexual health service guidance</t>
+          <t>Public health guidance</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>Đồng thuận, thân mật và thủ dâm</t>
+          <t>Nhịp sinh học, ánh sáng và áp lực ngủ</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Consent, intimacy and masturbation</t>
+          <t>Circadian timing, light and sleep pressure</t>
         </is>
       </c>
     </row>
     <row r="17" ht="86" customHeight="1" s="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>pelvic_women</t>
+          <t>sleep_habits</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>NHS — Urinary incontinence: non-surgical treatment</t>
+          <t>NHLBI — Healthy Sleep Habits</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>https://www.nhs.uk/conditions/urinary-incontinence/treatment/</t>
+          <t>https://www.nhlbi.nih.gov/health/sleep-deprivation/healthy-sleep-habits</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
@@ -5192,61 +5192,61 @@
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Đánh giá sàn chậu và tập có giám sát cho rò tiểu</t>
+          <t>Thói quen ngủ và lịch sinh hoạt</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>Pelvic-floor assessment and supervised training for leakage</t>
+          <t>Sleep habits and consistent schedules</t>
         </is>
       </c>
     </row>
     <row r="18" ht="86" customHeight="1" s="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>pelvic_women_relax</t>
+          <t>menopause</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Cambridge University Hospitals — Female pelvic floor muscle exercises</t>
+          <t>NHS — Symptoms of menopause and perimenopause</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>https://www.cuh.nhs.uk/patient-information/female-pelvic-floor-muscle-exercises/</t>
+          <t>https://www.nhs.uk/conditions/menopause-and-perimenopause/symptoms/</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Physiotherapy patient guidance</t>
+          <t>Public health guidance</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>Cần thả lỏng đầy đủ giữa các lần co cơ</t>
+          <t>Triệu chứng tiền mãn kinh và mãn kinh; khi cần khám</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>Full relaxation between pelvic-floor contractions</t>
+          <t>Perimenopause and menopause symptoms; seeking care</t>
         </is>
       </c>
     </row>
     <row r="19" ht="86" customHeight="1" s="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>menopause_care</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>NHS — Heavy periods</t>
+          <t>NHS — Menopause and perimenopause: treatment</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>https://www.nhs.uk/conditions/heavy-periods/</t>
+          <t>https://www.nhs.uk/conditions/menopause-and-perimenopause/treatment/</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -5256,413 +5256,413 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>Nhận biết chảy máu nhiều và các hướng điều trị</t>
+          <t>Thảo luận lợi ích và rủi ro điều trị triệu chứng mãn kinh</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Recognizing heavy menstrual bleeding and treatment options</t>
+          <t>Discussing benefits and risks of menopause symptom treatment</t>
         </is>
       </c>
     </row>
     <row r="20" ht="86" customHeight="1" s="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>cycle_hrv</t>
+          <t>libido</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Schmalenberger et al. (2019) — A Systematic Review and Meta-Analysis of Within-Person Changes in Cardiac Vagal Activity across the Menstrual Cycle</t>
+          <t>NHS — Low sex drive (loss of libido)</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/31726666/</t>
+          <t>https://www.nhs.uk/symptoms/loss-of-libido/</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>Systematic review and meta-analysis</t>
+          <t>Public health guidance</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>Biến đổi hoạt động phế vị theo chu kỳ ở cấp độ nhóm</t>
+          <t>Nhiều yếu tố ảnh hưởng ham muốn và chăm sóc theo nguyên nhân</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>Group-level cycle-related changes in cardiac vagal activity</t>
+          <t>Multiple influences on desire and cause-based care</t>
         </is>
       </c>
     </row>
     <row r="21" ht="86" customHeight="1" s="1">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>hrv</t>
+          <t>sexual_health</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Shaffer &amp; Ginsberg (2017) — An Overview of Heart Rate Variability Metrics and Norms</t>
+          <t>Devon Sexual Health (NHS) — Relationships and intimacy</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/29034226/</t>
+          <t>https://www.devonsexualhealth.nhs.uk/your-sexual-health/relationships-and-intimacy/</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Narrative review</t>
+          <t>Sexual health service guidance</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>Chỉ số HRV, bối cảnh đo và giới hạn so sánh</t>
+          <t>Đồng thuận, thân mật và thủ dâm</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>HRV metrics, recording context and comparability limits</t>
+          <t>Consent, intimacy and masturbation</t>
         </is>
       </c>
     </row>
     <row r="22" ht="86" customHeight="1" s="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>pulse</t>
+          <t>communication</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>American Heart Association — All About Heart Rate</t>
+          <t>Mallory et al. (2019) — Couples' Sexual Communication and Dimensions of Sexual Function: A Meta-Analysis</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>https://www.heart.org/en/health-topics/high-blood-pressure/the-facts-about-high-blood-pressure/all-about-heart-rate-pulse</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/30777780/</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Professional patient guidance</t>
+          <t>Meta-analysis of associations</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>Nhịp tim nghỉ, yếu tố ảnh hưởng và triệu chứng cần khám</t>
+          <t>Liên hệ giữa giao tiếp và chức năng tình dục; không chứng minh nhân quả</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>Resting pulse, influencing factors and warning symptoms</t>
+          <t>Association of communication and sexual function; not proof of causation</t>
         </is>
       </c>
     </row>
     <row r="23" ht="86" customHeight="1" s="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>activity</t>
+          <t>relationships</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>WHO — Physical activity</t>
+          <t>NHS — Maintaining healthy relationships and mental wellbeing</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>https://www.who.int/news-room/fact-sheets/detail/physical-activity</t>
+          <t>https://www.nhs.uk/every-mind-matters/lifes-challenges/maintaining-healthy-relationships-and-mental-wellbeing/</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Public health guideline summary</t>
+          <t>Public health guidance</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>Khuyến nghị vận động theo nhóm đối tượng</t>
+          <t>Giao tiếp, ranh giới và ứng phó bất đồng</t>
         </is>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>Activity recommendations by population</t>
+          <t>Communication, boundaries and managing disagreements</t>
         </is>
       </c>
     </row>
     <row r="24" ht="86" customHeight="1" s="1">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>overtraining</t>
+          <t>pelvic_men</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Meeusen et al. (2013) — Prevention, diagnosis, and treatment of the overtraining syndrome</t>
+          <t>North Tees and Hartlepool NHS — Pelvic Floor Exercises for Men</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/23247672/</t>
+          <t>https://www.nth.nhs.uk/resources/pelvic-floor-exercises-for-men/</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>Joint consensus statement</t>
+          <t>Physiotherapy patient guidance</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>Quá tải, chẩn đoán loại trừ và thiếu chỉ dấu đơn lẻ</t>
+          <t>Nhận biết, co và thả lỏng cơ sàn chậu nam</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>Overtraining, exclusion diagnosis and absence of a single marker</t>
+          <t>Identifying, contracting and relaxing male pelvic floor muscles</t>
         </is>
       </c>
     </row>
     <row r="25" ht="86" customHeight="1" s="1">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>sleep_habits</t>
+          <t>pelvic_relax</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>NHLBI — Healthy Sleep Habits</t>
+          <t>Royal Berkshire NHS (2024) — Pelvic floor strengthening and relaxation exercises for men</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>https://www.nhlbi.nih.gov/health/sleep-deprivation/healthy-sleep-habits</t>
+          <t>https://www.royalberkshire.nhs.uk/media/avwg3hls/pelvic-floor-strengthening-and-relaxation-exercises-for-men_jun24.pdf</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>Public health guidance</t>
+          <t>Physiotherapy patient guidance</t>
         </is>
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Thói quen ngủ và lịch sinh hoạt</t>
+          <t>Phối hợp tăng sức mạnh và thả lỏng; không kê bài siết cho tất cả</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>Sleep habits and consistent schedules</t>
+          <t>Strengthening and relaxation; not a prescription to tighten for everyone</t>
         </is>
       </c>
     </row>
     <row r="26" ht="86" customHeight="1" s="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>sleep_tech</t>
+          <t>pelvic_women</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Schutte-Rodin et al. (2021) — Evaluating consumer and clinical sleep technologies: an American Academy of Sleep Medicine update</t>
+          <t>NHS — Urinary incontinence: non-surgical treatment</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/34314344/</t>
+          <t>https://www.nhs.uk/conditions/urinary-incontinence/treatment/</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>Professional society review</t>
+          <t>Public health guidance</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>Giới hạn đánh giá và xác thực công nghệ theo dõi giấc ngủ</t>
+          <t>Đánh giá sàn chậu và tập có giám sát cho rò tiểu</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>Evaluation and validation limits of sleep technologies</t>
+          <t>Pelvic-floor assessment and supervised training for leakage</t>
         </is>
       </c>
     </row>
     <row r="27" ht="86" customHeight="1" s="1">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>iron</t>
+          <t>pelvic_women_relax</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>NHS — Iron deficiency anaemia</t>
+          <t>Cambridge University Hospitals — Female pelvic floor muscle exercises</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>https://www.nhs.uk/conditions/iron-deficiency-anaemia/</t>
+          <t>https://www.cuh.nhs.uk/patient-information/female-pelvic-floor-muscle-exercises/</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>Public health guidance</t>
+          <t>Physiotherapy patient guidance</t>
         </is>
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>Xét nghiệm thiếu máu và bổ sung sắt theo đánh giá</t>
+          <t>Cần thả lỏng đầy đủ giữa các lần co cơ</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>Anaemia testing and assessed iron replacement</t>
+          <t>Full relaxation between pelvic-floor contractions</t>
         </is>
       </c>
     </row>
     <row r="28" ht="86" customHeight="1" s="1">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>natural_fertility</t>
+          <t>pelvic_review</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>ASRM (2022) — Optimizing natural fertility: a committee opinion</t>
+          <t>Cohen et al. (2016) — The Role of Pelvic Floor Muscles in Male Sexual Dysfunction and Pelvic Pain</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>https://integration.asrm.org/globalassets/_asrm/practice-guidance/practice-guidelines/pdf/optimizing_natural_fertility.pdf</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/27872005/</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>Committee opinion</t>
+          <t>Clinical review</t>
         </is>
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>Thời điểm quan hệ, giới hạn dự đoán và khi đánh giá hiếm muộn</t>
+          <t>Quan hệ giải phẫu, chức năng sàn chậu và tiếp cận sinh học–tâm lý–xã hội</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>Intercourse timing, prediction limitations and fertility evaluation</t>
+          <t>Pelvic anatomy, function and a biopsychosocial approach</t>
         </is>
       </c>
     </row>
     <row r="29" ht="86" customHeight="1" s="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>ectopic</t>
+          <t>postpartum</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>NHS — Ectopic pregnancy: symptoms</t>
+          <t>ACOG — Exercise After Pregnancy</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>https://www.nhs.uk/conditions/ectopic-pregnancy/symptoms/</t>
+          <t>https://www.acog.org/womens-health/faqs/exercise-after-pregnancy</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Public health guidance</t>
+          <t>Professional patient guidance</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>Đau bụng, chảy máu, đau vai và chăm sóc khẩn</t>
+          <t>Trở lại vận động sau sinh tùy phương pháp sinh và biến chứng</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>Pain, bleeding, shoulder pain and urgent care</t>
+          <t>Postpartum return to activity by delivery and complications</t>
         </is>
       </c>
     </row>
     <row r="30" ht="86" customHeight="1" s="1">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>pregnancy</t>
+          <t>breathing</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>NHS — Common health problems in pregnancy</t>
+          <t>Zaccaro et al. (2018) — How Breath-Control Can Change Your Life: A Systematic Review on Psycho-Physiological Correlates of Slow Breathing</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>https://www.nhs.uk/pregnancy/common-symptoms/common-health-problems/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/30245619/</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Public health guidance</t>
+          <t>Systematic review</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>Triệu chứng thường gặp trong thai kỳ</t>
+          <t>Thở chậm, HRV và nghiên cứu không đồng nhất</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>Common pregnancy symptoms</t>
+          <t>Slow breathing, HRV and heterogeneous evidence</t>
         </is>
       </c>
     </row>
     <row r="31" ht="86" customHeight="1" s="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>pregnancy_exercise</t>
+          <t>hrv_measure</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>ACOG (2020) — Physical Activity and Exercise During Pregnancy and the Postpartum Period</t>
+          <t>Draghici &amp; Taylor (2016) — The physiological basis and measurement of heart rate variability in humans</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>https://www.acog.org/clinical/clinical-guidance/committee-opinion/articles/2020/04/physical-activity-and-exercise-during-pregnancy-and-the-postpartum-period</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/27680542/</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Committee guidance</t>
+          <t>Physiology review</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
         <is>
-          <t>Vận động thai kỳ, cá nhân hóa và dấu hiệu dừng tập</t>
+          <t>Cơ chế và giới hạn diễn giải HRV</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>Pregnancy activity, individualization and exercise warning signs</t>
+          <t>Mechanisms and interpretation limits of HRV</t>
         </is>
       </c>
     </row>
     <row r="32" ht="86" customHeight="1" s="1">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>intensity</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>CDC — Measuring Physical Activity Intensity</t>
+          <t>NHS — Heavy periods</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/physicalactivity/basics/measuring/index.html</t>
+          <t>https://www.nhs.uk/conditions/heavy-periods/</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
@@ -5672,145 +5672,657 @@
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>Talk test phân biệt vận động vừa và mạnh</t>
+          <t>Nhận biết chảy máu nhiều và các hướng điều trị</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t>Talk test for moderate and vigorous activity</t>
+          <t>Recognizing heavy menstrual bleeding and treatment options</t>
         </is>
       </c>
     </row>
     <row r="33" ht="86" customHeight="1" s="1">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>postpartum</t>
+          <t>cycle_hrv</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>ACOG — Exercise After Pregnancy</t>
+          <t>Schmalenberger et al. (2019) — A Systematic Review and Meta-Analysis of Within-Person Changes in Cardiac Vagal Activity across the Menstrual Cycle</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>https://www.acog.org/womens-health/faqs/exercise-after-pregnancy</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/31726666/</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>Professional patient guidance</t>
+          <t>Systematic review and meta-analysis</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>Trở lại vận động sau sinh tùy phương pháp sinh và biến chứng</t>
+          <t>Biến đổi hoạt động phế vị theo chu kỳ ở cấp độ nhóm</t>
         </is>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t>Postpartum return to activity by delivery and complications</t>
+          <t>Group-level cycle-related changes in cardiac vagal activity</t>
         </is>
       </c>
     </row>
     <row r="34" ht="86" customHeight="1" s="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>pcos</t>
+          <t>hrv</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Monash University — International evidence-based PCOS / PMOS guideline</t>
+          <t>Shaffer &amp; Ginsberg (2017) — An Overview of Heart Rate Variability Metrics and Norms</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>https://www.monash.edu/medicine/mchri/pcos/guideline</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/29034226/</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>International guideline</t>
+          <t>Narrative review</t>
         </is>
       </c>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>Chẩn đoán và chăm sóc toàn diện; cập nhật tên PMOS năm 2026</t>
+          <t>Chỉ số HRV, bối cảnh đo và giới hạn so sánh</t>
         </is>
       </c>
       <c r="F34" s="10" t="inlineStr">
         <is>
-          <t>Diagnosis and comprehensive care; PMOS terminology update in 2026</t>
+          <t>HRV metrics, recording context and comparability limits</t>
         </is>
       </c>
     </row>
     <row r="35" ht="86" customHeight="1" s="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>endometriosis</t>
+          <t>pulse</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>NHS — Endometriosis</t>
+          <t>American Heart Association — All About Heart Rate</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>https://www.nhs.uk/conditions/endometriosis/</t>
+          <t>https://www.heart.org/en/health-topics/high-blood-pressure/the-facts-about-high-blood-pressure/all-about-heart-rate-pulse</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>Public health guidance</t>
+          <t>Professional patient guidance</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>Triệu chứng, chẩn đoán và điều trị lạc nội mạc tử cung</t>
+          <t>Nhịp tim nghỉ, yếu tố ảnh hưởng và triệu chứng cần khám</t>
         </is>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>Endometriosis symptoms, assessment and treatment</t>
+          <t>Resting pulse, influencing factors and warning symptoms</t>
         </is>
       </c>
     </row>
     <row r="36" ht="86" customHeight="1" s="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>menopause_care</t>
+          <t>activity</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>NHS — Menopause and perimenopause: treatment</t>
+          <t>WHO — Physical activity</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>https://www.nhs.uk/conditions/menopause-and-perimenopause/treatment/</t>
+          <t>https://www.who.int/news-room/fact-sheets/detail/physical-activity</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
+          <t>Public health guideline summary</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>Khuyến nghị vận động theo nhóm đối tượng</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>Activity recommendations by population</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="86" customHeight="1" s="1">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Morton et al. (2018) — A systematic review, meta-analysis and meta-regression of the effect of protein supplementation on resistance training-induced gains in muscle mass and strength in healthy adults</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/28698222/</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>Systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>Protein và tập kháng lực ở người khỏe mạnh; không áp dụng trực tiếp cho bệnh thận</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>Protein with resistance training in healthy adults; not directly applicable to kidney disease</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="86" customHeight="1" s="1">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>liftmor</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Watson et al. (2018) — High-Intensity Resistance and Impact Training Improves Bone Mineral Density and Physical Function in Postmenopausal Women With Osteopenia and Osteoporosis: The LIFTMOR Randomized Controlled Trial</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/28975661/</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>Supervised randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>Tập có giám sát ở phụ nữ sau mãn kinh có khối lượng xương thấp</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>Supervised training in postmenopausal women with low bone mass</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="86" customHeight="1" s="1">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>overtraining</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Meeusen et al. (2013) — Prevention, diagnosis, and treatment of the overtraining syndrome</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/23247672/</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Joint consensus statement</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>Quá tải, chẩn đoán loại trừ và thiếu chỉ dấu đơn lẻ</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>Overtraining, exclusion diagnosis and absence of a single marker</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="86" customHeight="1" s="1">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>recovery</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Kellmann et al. (2018) — Recovery and Performance in Sport: Consensus Statement</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/29345524/</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Consensus statement</t>
+        </is>
+      </c>
+      <c r="E40" s="10" t="inlineStr">
+        <is>
+          <t>Phục hồi cần cá nhân hóa, gồm tải tập và áp lực cuộc sống</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>Individual recovery, training load and life demands</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="86" customHeight="1" s="1">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>sleep_tech</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Schutte-Rodin et al. (2021) — Evaluating consumer and clinical sleep technologies: an American Academy of Sleep Medicine update</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/34314344/</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>Professional society review</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>Giới hạn đánh giá và xác thực công nghệ theo dõi giấc ngủ</t>
+        </is>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>Evaluation and validation limits of sleep technologies</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="86" customHeight="1" s="1">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>sleep_stages</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>NHLBI — Sleep Phases and Stages</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhlbi.nih.gov/health/sleep/stages-of-sleep</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
           <t>Public health guidance</t>
         </is>
       </c>
-      <c r="E36" s="10" t="inlineStr">
-        <is>
-          <t>Thảo luận lợi ích và rủi ro điều trị triệu chứng mãn kinh</t>
-        </is>
-      </c>
-      <c r="F36" s="10" t="inlineStr">
-        <is>
-          <t>Discussing benefits and risks of menopause symptom treatment</t>
+      <c r="E42" s="10" t="inlineStr">
+        <is>
+          <t>NREM, REM và thay đổi theo tuổi</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>NREM, REM and age-related variation</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="86" customHeight="1" s="1">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>alcohol</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>WHO — Alcohol</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>https://www.who.int/news-room/fact-sheets/detail/alcohol</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>Public health evidence summary</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>Nguy cơ sức khỏe từ rượu; không có mức uống hoàn toàn không rủi ro</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>Alcohol-related health risks; no completely risk-free consumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="86" customHeight="1" s="1">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>iron</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Iron deficiency anaemia</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/iron-deficiency-anaemia/</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="inlineStr">
+        <is>
+          <t>Xét nghiệm thiếu máu và bổ sung sắt theo đánh giá</t>
+        </is>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>Anaemia testing and assessed iron replacement</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="86" customHeight="1" s="1">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>iron_bsg</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Snook et al. (2021) — British Society of Gastroenterology guidelines for the management of iron deficiency anaemia in adults</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/34497146/</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>Clinical practice guideline</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>Xác nhận thiếu sắt, diễn giải ferritin, tìm nguyên nhân và điều trị theo đáp ứng</t>
+        </is>
+      </c>
+      <c r="F45" s="10" t="inlineStr">
+        <is>
+          <t>Iron deficiency confirmation, ferritin interpretation, cause investigation and response-based treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="86" customHeight="1" s="1">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>natural_fertility</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>ASRM (2022) — Optimizing natural fertility: a committee opinion</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>https://integration.asrm.org/globalassets/_asrm/practice-guidance/practice-guidelines/pdf/optimizing_natural_fertility.pdf</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>Committee opinion</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="inlineStr">
+        <is>
+          <t>Thời điểm quan hệ, giới hạn dự đoán và khi đánh giá hiếm muộn</t>
+        </is>
+      </c>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>Intercourse timing, prediction limitations and fertility evaluation</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="86" customHeight="1" s="1">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>pregnancy</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Common health problems in pregnancy</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/pregnancy/common-symptoms/common-health-problems/</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
+        <is>
+          <t>Triệu chứng thường gặp trong thai kỳ</t>
+        </is>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>Common pregnancy symptoms</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="86" customHeight="1" s="1">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>pregnancy_exercise</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>ACOG (2020) — Physical Activity and Exercise During Pregnancy and the Postpartum Period</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>https://www.acog.org/clinical/clinical-guidance/committee-opinion/articles/2020/04/physical-activity-and-exercise-during-pregnancy-and-the-postpartum-period</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>Committee guidance</t>
+        </is>
+      </c>
+      <c r="E48" s="10" t="inlineStr">
+        <is>
+          <t>Vận động thai kỳ, cá nhân hóa và dấu hiệu dừng tập</t>
+        </is>
+      </c>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>Pregnancy activity, individualization and exercise warning signs</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="86" customHeight="1" s="1">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>fitness</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>Ross et al. (2016) — Importance of Assessing Cardiorespiratory Fitness in Clinical Practice</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/27881567/</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>AHA scientific statement</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="inlineStr">
+        <is>
+          <t>Thể lực tim phổi và đánh giá nguy cơ sức khỏe</t>
+        </is>
+      </c>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
+          <t>Cardiorespiratory fitness and health risk assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="86" customHeight="1" s="1">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>intensity</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>CDC — Measuring Physical Activity Intensity</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/physicalactivity/basics/measuring/index.html</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E50" s="10" t="inlineStr">
+        <is>
+          <t>Talk test phân biệt vận động vừa và mạnh</t>
+        </is>
+      </c>
+      <c r="F50" s="10" t="inlineStr">
+        <is>
+          <t>Talk test for moderate and vigorous activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="86" customHeight="1" s="1">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>pcos</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>Monash University — International evidence-based PCOS / PMOS guideline</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>https://www.monash.edu/medicine/mchri/pcos/guideline</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>International guideline</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>Chẩn đoán và chăm sóc toàn diện; cập nhật tên PMOS năm 2026</t>
+        </is>
+      </c>
+      <c r="F51" s="10" t="inlineStr">
+        <is>
+          <t>Diagnosis and comprehensive care; PMOS terminology update in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="86" customHeight="1" s="1">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>endometriosis</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>NHS — Endometriosis</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/endometriosis/</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>Public health guidance</t>
+        </is>
+      </c>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>Triệu chứng, chẩn đoán và điều trị lạc nội mạc tử cung</t>
+        </is>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
+        <is>
+          <t>Endometriosis symptoms, assessment and treatment</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F36"/>
+  <autoFilter ref="A1:F52"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -5847,6 +6359,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId51"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>